<commit_message>
build-analysis: Examples & mock map tab — worked example per gap + final-mock mapping + look-change verdict (founder order: no UX change without seeing the new screen)
Verified against mockups/final: path-ahead + grouping toggle ARE drawn in
networth-v7 (build = conform); winners 1+1 matches invest-v7 (doc's 3+2 is
stale); dollar-first items shown in home-v2; income line/range strip/source
chips in NO final mock -> PARKED behind new mocks.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -9,11 +9,12 @@
   <sheets>
     <sheet name="How to read" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="SUMMARY — read me first" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="UX design v1.1" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Design — Invest·CF·Plan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Design — Home·Net worth" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Strategy &amp; data lineage" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="PRD v1.1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Examples &amp; mock map" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="UX design v1.1" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Design — Invest·CF·Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Design — Home·Net worth" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Strategy &amp; data lineage" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="PRD v1.1" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39,7 +40,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -49,6 +50,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E1F5EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4EAD8"/>
       </patternFill>
     </fill>
   </fills>
@@ -64,7 +70,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -73,6 +79,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -828,6 +837,1671 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Gap (source tab)</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>A concrete example — before → after</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Screen(s)</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>In a final approved mock?</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Look change?</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>What you would actually see · my commitment</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr"/>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>— GROUP A · ACCURACY (candidates for Build 46) —</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr"/>
+      <c r="D2" s="4" t="inlineStr"/>
+      <c r="E2" s="4" t="inlineStr"/>
+      <c r="F2" s="4" t="inlineStr"/>
+      <c r="G2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>SS adoption odds (PRD #2)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Your statement says $2,600/mo at 67. You adopt claim-at-62 → the real check is ~$1,820. The SS screen showed you "74% chance" for that choice; Home and Plan then quietly compute with the full $2,600 and show ~79%. After the fix, every screen says 74%.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Home · Plan hub · SS timing</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>n/a (numbers, not layout)</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Screens look pixel-identical — only the disagreement disappears. No mock needed; an agreement test pins all three screens to one number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Unpriced holding shows $0 (Invest #2)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Your LCTX has no live price feed yet. Invest list today: "LCTX … $0". After: "LCTX … $1,132" with the small words "what you paid" beneath — the same honest treatment its own detail page already uses.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Invest list</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>v7 mock shows priced rows only</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>TINY</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>One number and three small words change on an existing row. I will show you the exact row rendering before it builds if you want — say "show me" and it is in the next mock batch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Insight sheet escapes the mask (PRD #6)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Eye ON (balances hidden): the card says "••••" — but tap it and the pop-up sheet reads "You can still contribute $9,200 this year" in plain dollars. After: the sheet shows "•••• this year" like everywhere else.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Home insights pop-up</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Visible only when you hide balances; then it simply masks like every other surface. No mock needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>— GROUP B · TRUST &amp; DRIFT TRAPS (fix soon) —</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Bond/alt sales skip the ledger (Home·NW #20)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Sell your $10,000 CD → the balance drops, but the account's Activity shows nothing. A month later there is no way to see where $10,000 went. After: a SELL row appears in Activity, exactly like stock sales already do.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Bond/Alt editors · Account detail activity</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Account-detail FINAL shows the activity list</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>No layout change — rows simply start appearing in the existing, approved activity list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Market-average math duplicated (Strategy #5)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Home and Invest both say "the market: up 8.2%" because two identical copies of the formula exist. Edit one copy alone someday and the two screens silently disagree. The fix merges them into one shared calculation.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Home · Invest</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Invisible. An agreement test pins both screens to the one helper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Equity vesting months disagree (PRD #4)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>You add $24,000/yr of stock vesting in March + September. Cash flow correctly shows $12,000 in Mar and $12,000 in Sep — the income engine's year view still parks all $24,000 in December.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Income detail vs Cash flow</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>No layout change — the December lump just moves to the months it really lands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Adoption sheet thinner than contract (Design ICP #25)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Today, adopting claim-62 shows two lines ("Claim age 67 → 62 · Check $2,600 → $1,820") and a Confirm. The approved design also shows "Will my money last: 84% → 74%", "You'll see this on: Home, Plan, Cash flow", and two EQUAL-weight buttons.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>The Use-this-plan sheet (all scenarios)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Not drawn in any final mock</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>PARKED. I will mock the full sheet (rich + minimal states) and build only after your approve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>— GROUP C · APPROVED BUT NEVER BUILT (your triage) —</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>"Your path ahead" row on Net worth (Home·NW #15)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Under the trend chart, one calm line: "Your path ahead (from your Plan): on course for ~$310,000 by 67 ›". Today: nothing there.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Net worth</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>YES — drawn in networth-v7 FINAL</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>YES (to the approved picture)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>The new look already exists — open networth-v7-hifi-FINAL and you are looking at it. Building = making the app match your approved mock. Zero new design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>NW grouping toggle (Home·NW #13)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Above the class list: [By class] [By institution] [By type]. Tap "By institution" → your two E*TRADE entries roll up under one E*TRADE header. Today: only the class view exists.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Net worth</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>YES — drawn in networth-v7 FINAL</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>YES (to the approved picture)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Same as above: your approved mock IS the picture. No new design needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Source chips on NW rows (Home·NW #14)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Each account row would wear a small pill: "🔗 Connected · Jul 22" / "📄 Imported · Jun 12". Today the sub-line text carries it only in the setup path.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Net worth rows</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>NO — not in v7</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>PARKED — mock first, then your call.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Return breakdown on Invest (Design ICP #3)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Under YOUR RETURN +$1,860: "price change +$1,540 · dividends +$260 · interest +$60" — adding up to the headline.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Invest</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>NO — not in v7</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>PARKED — mock first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Per-number staleness stamps (Home·NW #6)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>E*TRADE hasn't updated for 3 days → the hero gains a line "as of Jul 21 (E*TRADE part)".</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Home · Net worth</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>PARKED — mock first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Loading / offline states (Home·NW #4)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Airplane mode → today the numbers just render with no hint. Approved: "We couldn't refresh just now — showing your numbers from Jul 21. [Try again]".</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>PARKED — mock first (it is one banner line, but you will see it drawn).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>SS compare for ages 67-69 (Design ICP #22)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>You are 68: today the compare greys out 62 and 67 as "passed" and only 70 is real — there is no "claim now" option. After: the rows become "Claim now (68): $2,710/mo" vs "Wait to 70: $3,220/mo".</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>SS timing</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Screen pattern approved; this state not drawn</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>TINY</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Same approved table, different rows for this age group. I will include the 68-year-old state in the next mock batch for your eyes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Goals starter examples (Design ICP #23)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Goals empty state today: "No goals yet — add one on the Goals screen." Approved: four grey example goals (New roof $18k · Trip $6k · Car $30k · Gift $10k) + "Add your own".</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Multi-goal</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>PARKED — mock first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Roth banner + save + action item (Design ICP #24)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>The Roth screen today has no "You're trying things out — nothing is saved" banner (every other scenario screen has it), no Save-scenario, and adopting creates no "Convert by Dec 31" item on the Plan hub.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Roth · Plan hub</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Banner exists on sibling screens (approved element)</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>TINY-YES</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>The banner = the exact approved element from sibling screens (conforming). The hub action item is new — mock first for that part.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Look-back extras (Design ICP #9)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>"What if I'd put $10,000 in NVDA a year ago" exists — but no "…or left it in cash" chip, no 6-month window, no reset link, no stale-price note.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Look-back</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>PARKED — mock first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Matured bond banner (Design ICP #8)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Your CD matured Jun 30. Today it still sits listed as a bond with "(matured)". Approved: a banner "This CD matured — record what happened [Record payoff]".</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Account detail (bonds)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>TINY-YES</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>PARKED — mock first (one banner).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Bonds-only hero (Design ICP #5)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>A user holding only CDs opens Invest and gets no summary at all. Approved: "Total value $84,000 · returns appear when prices or your reported return exist."</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Invest</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>NO (mock shows priced state)</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>TINY-YES</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>PARKED — mock first (empty-state rule: you see every data state).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Invest empty state + import door (Design ICP #4)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Brand-new user: today one door ("＋ Add a holding"). Approved: the sentence + TWO doors (add by hand / import from a file).</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Invest day-one</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>NO — v7 has no empty state</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>TINY-YES</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>PARKED — mock first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Reduce-motion (UX #17)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>iPhone Settings → Reduce Motion ON: today the app still animates count-ups and slides. After: those users get instant, still screens.</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>App-wide</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Nothing changes for you — only for users who asked their phone for less motion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Disconnect on the account page (Home·NW #21)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>To unlink E*TRADE today you must find Settings → connections. Approved: the account's own page carries [Disconnect] with "your numbers and history stay".</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Account detail</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Not drawn in account-detail FINAL</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>TINY-YES</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>PARKED — micro-mock first. Note the wording depends on your keep-vs-delete decision (Group E).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Richer duplicate matching (Home·NW #18)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>You import a file containing the E*TRADE account you already track. Today's match keys are coarse (institution+kind); the approved rule also matches name / last-4 / balance-within-10% and suffixes "keep both" twins.</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Connect/import merge</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Invisible logic — just fewer duplicate-account accidents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Treasury kind (Home·NW #19)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Adding a T-bill today: you pick "Bond/CD" and it is treated right only if the word "treasury" is in the label. Approved: an explicit Treasury choice in the editor.</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Add-account/bond editor</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>TINY</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>One extra chip in an existing picker — included in the next mock batch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Undated-value nudge (Design ICP #29)</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>An account whose value has no date today shows nothing. Approved: "value date unknown — confirm it once", same style as the existing "still right?" nudge.</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Account detail</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Same style as approved nudge</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>TINY</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>One line in the approved nudge style.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Month switcher vs Debts tab (Design ICP #16)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Flip Cash flow back to June: This month / Income / Spending all time-travel — Debts silently keeps showing today. Either Debts respects the month or it honestly says "Debts are always current".</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Cash flow · Debts tab</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Mock does not address it</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>TINY</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Your pick of the two behaviors; one is a label, the other is real month-travel. Both described, neither built until you choose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Investment-income line (Design ICP #14)</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>THIS MONTH today: Salary $6,200. Approved: also "Dividends &amp; interest · $310" as its own labeled line when it exists.</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Cash flow · This month</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>NO — not in cashflow-4tabs FINAL</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>TINY-YES</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>PARKED — mock first (one line, but it changes your approved This-month card).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Will-it-last range strip (Design ICP #13)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Strip today: "84% · estimate". Approved: "84% — holds 71-95% across bad-to-good markets".</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Cash flow strip · Will-it-last</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>TINY</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>A few words appended to an existing line — in the next mock batch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Plan-hub small honesty rows (Design ICP #19-21)</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Claim-window date badge on the SS row ("you can claim from Sep 2026") · reopened scenario shows "was 79% saved, 78% today" · Revert opens the same field-diff sheet instead of a bare alert.</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Plan hub</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>TINY-YES</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>PARKED — one combined micro-mock for the three.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Will-it-last detail depth (Design ICP #26)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Approved: a drawn band chart, ranked "what moves it most" ("spend $500 less → 89%"), a sharpen meter, inline edits. Today: text range + unranked drivers + link-outs.</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Will-it-last detail</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>NO — never drawn hi-fi</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>YES (biggest)</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>PARKED — this is the largest unbuilt piece. Mock first, and you decide pre- vs post-launch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr"/>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>— GROUP D · COPY &amp; POLISH SWEEP —</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr"/>
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Bare acronyms (UX #18)</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>"12.99% APR" → "12.99% yearly interest (APR)" · "YTM 4.1%" → "Yield to maturity: 4.1%" · glossary title "RMD" → "Required withdrawals (RMD)".</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Budget · Bonds · glossary</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>TINY</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Words only, layouts identical. Also your standing no-acronyms rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Nest-egg info dot verbatim (Design ICP #12)</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>You approved: "…The amount shown represents the incremental wealth… An estimate, not a promise." The shipped text drifted to wonkier phrasing. After: your words, letter for letter.</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Look-ahead info dot</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Your copy IS the approval</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>TINY</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Restores your exact approved text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Dollar-first what-needs-you (Home·NW #1)</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>"42% of your investable money is in one account" → "$71,000 (42%) sits in one account" — dollars first, as your approved Home mock shows.</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>YES — home-v2 mock shows dollar-first</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>TINY</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Conforms to your approved mock — open home-v2 and you are looking at it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Wording unifications (UX #10/#13, Design ICP #17)</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Ten "estimate" chip variants → one; three "trying it out" banners → one wording; Debts empty line and /budget landing aligned to the approved sentences.</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Various</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Approved sentences exist</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>TINY</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Same layouts, one consistent voice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Tap targets (UX #5)</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Some rows/links are 32-40pt tall vs the 44/52 rule — fingers miss them. Fix: the same rows, a touch taller.</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>NW rows · sheet links</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Spacing only</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>TINY</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Nothing moves or changes words; rows get slightly taller. A ratchet test keeps it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Paycheck card details (Home·NW #10)</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>"This year $71,600" → "~$71,600" · button "See all 12 months" → "See July's paycheck".</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Home paycheck card</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Doc-specified</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>TINY</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Words only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Masked money spoken as "hidden" (Home·NW #8)</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>A screen reader today reads "••••" as dots; after, it says "hidden".</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>App-wide</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Spoken only; nothing visual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr"/>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>— GROUP E · YOUR OPEN DECISIONS (examples of each option) —</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr"/>
+      <c r="D43" s="4" t="inlineStr"/>
+      <c r="E43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>17pt money floor (UX #3)</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Winners table RETURN column today: 10.5pt. At 17pt the same column is ~60% larger — on your approved v7 table that means fewer columns fit or rows wrap.</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>All dense tables</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>v7 tables approved at current sizes</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>YES if adopted</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>If you choose 17: I mock the affected tables FIRST so you see the wrapping trade-off before anything changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Empty-odds strip (Home·NW #3)</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Option A (your Jul-15 approval): locked gauge "Sample: 84%…". Option B (the later mock): "Answer 3 quick questions in Plan to see your odds ›".</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>BOTH approved, dates conflict</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Pick one</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Both already exist as pictures — say A or B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Disconnect promise (Home·NW #17)</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Option A: "Disconnect — your numbers and history stay" (doc). Option B: "Disconnect — we delete the connection's data" (shipped consent).</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Consent + Settings + account page</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Words + behavior</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Pick the promise; copy and behavior then align everywhere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Legacy modules in v1 (Strategy #4)</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Estate, Insurance, Tax organizer, Job safety, Credit are reachable today. Keep = more value, more to test (they are in your 97-row walk). Hide = tighter launch.</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Menu / routes</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Not in FCC docs</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Pick</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Either way is one small change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Price provider (Strategy #3)</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Your "vs the market" hook rides a free unofficial feed that can break without notice. The keyed-provider seam is ready — the pick (Tiingo is ruled out) is yours.</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Invest · NW history</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Engine only; unblocks dividends/total-return and live LCTX pricing (kills the $0 class for good).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Color palettes (UX #1-2)</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Example: Cash is teal on Net worth but a different color in the Invest chart; the doc's validated palettes were never adopted.</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Charts app-wide</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Mocks show shipped colors</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>YES if adopted</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>If you want the validated palettes: recolored mocks first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Emergency cushion card (Home·NW #16)</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Doc: a cushion card below the fold ("4.2 months of essentials"). Your final v7 mock dropped it, and the code never renders it.</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Net worth</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Absent from v7 FINAL</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Pick</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Say "drop" (doc edit + dead code removed) or "build" (mock first).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1476,7 +3150,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2460,7 +4134,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3204,7 +4878,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3588,7 +5262,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Build-status column extended to ALL tabs of the master audit file (founder request)
The five document tabs (UX / Design x2 / Strategy+lineage / PRD) gain column G:
99 rows each tagged PROPOSED (with walk row) / PARKED / NEXT WALK ROUND /
DECIDED / OPEN / DOC REFRESH / DELIVERED / NO ACTION / DEVICE CHECK /
POST-LAUNCH. Rows cite their action item so tabs can never disagree.
Surfaced 4 additional OPEN founder picks that were not in the action list:
month bars vs rows (UX 6), donut slice labels (UX 7), winners 1+1 vs 3+2
(ICP 1), plan-incomplete nudge gate (PRD 7). How-to-read legend updated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,6 +70,11 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0044546A"/>
+      <sz val="10.5"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -101,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -130,6 +135,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -552,15 +560,15 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
+    <row r="6" ht="90" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Column H — Build status (added 2026-07-28)</t>
+          <t>Build status column (added 2026-07-28, extended to every tab 2026-07-29)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Your one-master-file request: column H on "Examples &amp; mock map" says for every item whether it is PROPOSED for Build 46 (with its row number in the walk workbook), PARKED at the mock gate, queued for the NEXT walk round, DECIDED (with your call), or OPEN for your pick. As items build, I update the cell to "BUILT — Build N" the same day. This file is the monitor; build46-item-walk-v1-2026-07-28.xlsx is just the approval form for the current batch.</t>
+          <t>Your one-master-file request: EVERY tab now carries a Build status column (H on Examples &amp; mock map, G on the five document tabs). It says for each row: PROPOSED for Build 46 (with its row in the walk workbook) · PARKED at the mock gate · NEXT WALK ROUND (no picture needed, proposed after this batch) · DECIDED (your call, dated) · OPEN (a pick still yours to make) · DOC REFRESH (paper edit only, nothing to build) · DELIVERED · NO ACTION (deliberate, founder-known deviation) · DEVICE CHECK · POST-LAUNCH. Rows that map to an action item cite it, so the tabs can never disagree. As items build I update the cells to "BUILT — Build N" the same day. This file is the master monitor; build46-item-walk-v1-2026-07-28.xlsx is just the approval form for the current batch.</t>
         </is>
       </c>
     </row>
@@ -2790,7 +2798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2799,6 +2807,7 @@
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2832,6 +2841,11 @@
           <t>What it means for you / recommended action</t>
         </is>
       </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Build status — proposed vs built (added 2026-07-29; kept current)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="64" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -2862,6 +2876,11 @@
           <t>The app is colorblind-safe in practice (word + icon everywhere), but the palette you validated was never adopted. Decide: adopt the doc palette, or bless the shipped one and update the doc.</t>
         </is>
       </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-07-28 — adopt the validated palettes; recolored mocks first (action item 43)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="64" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -2892,6 +2911,11 @@
           <t>Same-class-same-color everywhere is the point of a fixed palette. Recommend unifying on ONE keyed palette (either set) — small change, real consistency win.</t>
         </is>
       </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-07-28 — adopt the validated palettes; recolored mocks first (action item 43)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="64" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -2922,6 +2946,11 @@
           <t>This is your explicitly parked decision (17pt floor vs dense tables). Nothing enforces 17 until you decide. If you pick 17, I raise the ratchet and sweep every money size in one pass.</t>
         </is>
       </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-07-28 — dense tables keep approved compact sizes; question closed, nothing to build (action item 38)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="64" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -2952,6 +2981,11 @@
           <t>Visual drift risk, not a correctness bug. Worth one consolidation pass after launch-critical work.</t>
         </is>
       </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — one shared hero component at today’s sizes; invisible consolidation</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -2982,6 +3016,11 @@
           <t>A 65+ audience feels small targets. Recommend a one-pass sweep + a ratchet test so it never regresses.</t>
         </is>
       </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 13 · your verdict pending (action item 35)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="64" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -3012,6 +3051,11 @@
           <t>The shipped rows are readable but not what the doc drew. Decide which you prefer — the cash-flow surface was approved later from mocks, so the DOC may be the stale one here.</t>
         </is>
       </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>OPEN — your pick, brought drawn: keep the shipped month rows (doc edit) or the doc’s paired bars with a now-marker (mock batch)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -3042,6 +3086,11 @@
           <t>Legend + spoken sentence is honest but not the mandated direct labeling. Small change if you want it.</t>
         </is>
       </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>OPEN — your pick, brought drawn: keep legend + spoken sentence (doc edit) or direct slice labels (mock batch)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="2" t="n">
@@ -3072,6 +3121,11 @@
           <t>Words are honest; the drawn band was the approved visual. Decide keep-words vs draw-band.</t>
         </is>
       </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — the drawn band rides the will-it-last detail mock (action item 30)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="64" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -3102,6 +3156,11 @@
           <t>You approved the invest-v7 TABLE design on 2026-07-19 (mockups/final/invest-v7) which replaced the bar idea. The doc row predates it; the doc needs the edit, not the code.</t>
         </is>
       </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>DOC REFRESH — you approved the v7 table (2026-07-19); paper edit only, nothing to build</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="2" t="n">
@@ -3132,6 +3191,11 @@
           <t>Consistency-of-honesty matters to trust. Recommend one shared chip component; mechanical change.</t>
         </is>
       </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 12 · one shared estimate chip (action item 34)</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -3162,6 +3226,11 @@
           <t>Shipped version is quieter than specced. Decide whether the pill + tap-sheet is still wanted.</t>
         </is>
       </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — pill + tap-sheet rides the source-chips mock (action item 10)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="2" t="n">
@@ -3192,6 +3261,11 @@
           <t>The doc wanted no steering pressure on a money decision. One-line style change if you confirm.</t>
         </is>
       </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — folded into the full adoption-sheet mock (action item 7)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="2" t="n">
@@ -3222,6 +3296,11 @@
           <t>Unify to one string constant + add the missing Roth banner. Small, real.</t>
         </is>
       </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 12 · one wording; the missing Roth banner itself = action item 16, next walk round</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="64" customHeight="1">
       <c r="A15" s="2" t="n">
@@ -3252,6 +3331,11 @@
           <t>Both deviations protect honesty/accessibility and were surfaced when built. Doc should record them.</t>
         </is>
       </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>NO ACTION — deliberate, founder-known deviation (honesty/accessibility); recorded in the doc refresh</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="2" t="n">
@@ -3282,6 +3366,11 @@
           <t>Your later decision wins; the doc needs the edit.</t>
         </is>
       </c>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>DOC REFRESH — your 2026-07-16 reversal wins; paper edit only</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="2" t="n">
@@ -3312,6 +3401,11 @@
           <t>Screen-reader coverage is real but ad-hoc. Either add the label to the shared component or re-word the doc rule to match the per-card pattern.</t>
         </is>
       </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — spoken label on the shared money component + a guard test; invisible</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -3342,6 +3436,11 @@
           <t>Real accessibility gap for a 65+ audience. Moderate effort; recommend post-Build-46 but before public launch.</t>
         </is>
       </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — respects the phone’s reduce-motion setting; invisible (action item 21)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="2" t="n">
@@ -3372,6 +3471,11 @@
           <t>Also violates your standing no-acronyms rule. Quick sweep: "interest rate (APR)" spelled once, "yield to maturity", "required withdrawals (RMD)".</t>
         </is>
       </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 10 · your verdict pending (action item 31)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -3402,6 +3506,11 @@
           <t>The doc disagrees with itself; pick one sentence and align the doc.</t>
         </is>
       </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>DOC REFRESH — the doc disagrees with itself; code matches the Components sentence; one-line paper fix</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="64" customHeight="1">
       <c r="A21" s="2" t="n">
@@ -3430,6 +3539,11 @@
       <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Large-text survival, 375pt fit and thumb-reach are device-review items no code audit can prove — they belong on your device walk.</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>— coverage note · large-text, 375pt fit and thumb reach ride your device walk</t>
         </is>
       </c>
     </row>
@@ -3444,7 +3558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3453,6 +3567,7 @@
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3486,6 +3601,11 @@
           <t>What it means for you / recommended action</t>
         </is>
       </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Build status — proposed vs built (added 2026-07-29; kept current)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -3516,6 +3636,11 @@
           <t>Decide: keep the calmer 1+1 (then the doc gets edited) or show the 3+2 you specced. Ranking by contribution is the more meaningful ordering either way.</t>
         </is>
       </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>OPEN — your pick, brought drawn: keep the calmer 1 leader + 1 laggard (doc edit) or the doc’s 3+2 ranked by contribution (mock batch)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="64" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -3546,6 +3671,11 @@
           <t>A wrong $0 is the trust-killer class. Recommend fixing before Build 46 ships: fall back to cost basis with the honest "what you paid" word on the list row too.</t>
         </is>
       </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 2 · your verdict pending (action item 2)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -3576,6 +3706,11 @@
           <t>Meaningful transparency feature from the approved doc that never got built on the main screen.</t>
         </is>
       </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — mock first (action item 11)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -3606,6 +3741,11 @@
           <t>The import door matters on day one. Small fix.</t>
         </is>
       </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — mock first (action item 20)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -3636,6 +3776,11 @@
           <t>A real user state (CD-heavy 65+) that sees a half-empty screen. Worth fixing.</t>
         </is>
       </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — mock first (action item 19)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -3666,6 +3811,11 @@
           <t>Mild but confusing when you switch periods. Small fix.</t>
         </is>
       </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — detail mirrors the selected period; small conformance, no new picture</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -3696,6 +3846,11 @@
           <t>Small reach-through interaction never wired.</t>
         </is>
       </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — tap scrolls to the holding; small interaction, no new picture</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="2" t="n">
@@ -3726,6 +3881,11 @@
           <t>Matters for CD-heavy users; the money sits mislabeled after maturity.</t>
         </is>
       </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — mock first, one banner (action item 18)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -3756,6 +3916,11 @@
           <t>The "what if I'd stayed in cash" comparison was a distinctive approved idea; still unbuilt.</t>
         </is>
       </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — mock first (action item 17)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="2" t="n">
@@ -3786,6 +3951,11 @@
           <t>The PRD-approved progressive-tax work (Jul 15) superseded this row. Doc edit only.</t>
         </is>
       </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>DOC REFRESH — code is better than the doc (your progressive-tax approval); paper edit only</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -3816,6 +3986,11 @@
           <t>The extra gates were approved with the lookahead redesign. Doc edit.</t>
         </is>
       </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>DOC REFRESH — the extra honest gates were approved with the look-ahead redesign; paper edit only</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="2" t="n">
@@ -3846,6 +4021,11 @@
           <t>Your verbatim copy was the approval. Restore it word-for-word.</t>
         </is>
       </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 11 · your verdict pending (action item 32)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="2" t="n">
@@ -3876,6 +4056,11 @@
           <t>The range is the honesty device. Small copy addition.</t>
         </is>
       </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — a few words, shown drawn first (action item 28)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="2" t="n">
@@ -3906,6 +4091,11 @@
           <t>Matters most for the 55-70 audience living partly on investment income.</t>
         </is>
       </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — mock first (action item 27)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="2" t="n">
@@ -3936,6 +4126,11 @@
           <t>Honesty deviation, surfaced when built. The doc should record it so it stops reading as a gap.</t>
         </is>
       </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>NO ACTION — deliberate honesty deviation (the odds model is not order-aware); recorded in the doc refresh</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="2" t="n">
@@ -3966,6 +4161,11 @@
           <t>Debts is genuinely month-less today; either wire it or say so on the tab.</t>
         </is>
       </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>OPEN — your pick of the two behaviors, brought drawn (action item 26)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="64" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -3996,6 +4196,11 @@
           <t>Your later decision wins, but the doc claims it in TWO places (spec + build-status) — both need the edit. Flagging because the status column asserting "built" for something absent is exactly the doc-vs-truth risk you called out.</t>
         </is>
       </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>DOC REFRESH — your 2026-07-16 reversal wins, in both places the doc claims it; paper edit only</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="2" t="n">
@@ -4026,6 +4231,11 @@
           <t>Two 1-line fixes; the redirect landing is defensible — your call.</t>
         </is>
       </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 12 · your verdict pending (action item 34)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -4056,6 +4266,11 @@
           <t>Small; the date is the hook that makes the row feel personal.</t>
         </is>
       </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — one combined micro-mock for the three Plan-hub rows (action item 29)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="2" t="n">
@@ -4086,6 +4301,11 @@
           <t>The was/now contrast is an honesty feature worth building.</t>
         </is>
       </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — same combined micro-mock (action item 29)</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="2" t="n">
@@ -4116,6 +4336,11 @@
           <t>Symmetry of consent: reverting deserves the same clarity as adopting.</t>
         </is>
       </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — same combined micro-mock (action item 29)</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="2" t="n">
@@ -4146,6 +4371,11 @@
           <t>Real cohort in your 55-70 target. Recommend fixing.</t>
         </is>
       </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — approved table pattern incl. the 68-year-old state; no new picture (action item 14)</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="2" t="n">
@@ -4176,6 +4406,11 @@
           <t>Starter examples teach the feature; small build.</t>
         </is>
       </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — mock first (action item 15)</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="2" t="n">
@@ -4206,6 +4441,11 @@
           <t>The banner is also a UX-doc rule; the action item is the follow-through that makes adoption real.</t>
         </is>
       </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — conforming banner + save + dated action item (action item 16)</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="48" customHeight="1">
       <c r="A26" s="2" t="n">
@@ -4236,6 +4476,11 @@
           <t>This sheet is the app's biggest consent moment and it is thinner than its approved contract. Recommend prioritizing.</t>
         </is>
       </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — full adoption-sheet mock, rich + minimal states (action item 7)</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="2" t="n">
@@ -4266,6 +4511,11 @@
           <t>The flagship "honest odds" screen shipped at half its approved depth. Decide how much to build pre- vs post-launch.</t>
         </is>
       </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — the biggest unbuilt piece; mock first, you decide pre- vs post-launch when you see it (action item 30)</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="2" t="n">
@@ -4296,6 +4546,11 @@
           <t>Code is AHEAD of the doc. The status column needs one refresh pass.</t>
         </is>
       </c>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>DOC REFRESH — code is ahead of the doc; the nine statuses get one refresh pass</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="32" customHeight="1">
       <c r="A29" s="2" t="n">
@@ -4326,6 +4581,11 @@
           <t>One-line suppression rule.</t>
         </is>
       </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — one-line suppression rule; invisible</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="32" customHeight="1">
       <c r="A30" s="2" t="n">
@@ -4356,6 +4616,11 @@
           <t>Quiet data-quality hole; small fix.</t>
         </is>
       </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — one line in the approved nudge style (action item 25)</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="64" customHeight="1">
       <c r="A31" s="2" t="n">
@@ -4386,6 +4651,11 @@
           <t>Included so you know the audit was checked, not just collected. Claims that failed verification were dropped.</t>
         </is>
       </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>— audit-integrity note · claim refuted by hand-check, nothing to build</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="64" customHeight="1">
       <c r="A32" s="2" t="n">
@@ -4414,6 +4684,11 @@
       <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Differences listed above are the complete set that survived verification.</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>— coverage note</t>
         </is>
       </c>
     </row>
@@ -4428,7 +4703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4437,6 +4712,7 @@
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4470,6 +4746,11 @@
           <t>What it means for you / recommended action</t>
         </is>
       </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Build status — proposed vs built (added 2026-07-29; kept current)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -4500,6 +4781,11 @@
           <t>Dollar-first was the approved persuasion device and one item breaks the facts-never-instructions rule. Small copy/math fix, real impact.</t>
         </is>
       </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 9 · picture already approved, home-v2 (action item 33)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -4530,6 +4816,11 @@
           <t>The shared-selector approach is stronger than the doc's (numbers can never disagree). Doc edit.</t>
         </is>
       </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>DOC REFRESH — code is stronger than the doc (one shared selector); paper edit only</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -4560,6 +4851,11 @@
           <t>Your two approvals conflict by date. Pick one: sample gauge or the 3-questions line; I align the loser.</t>
         </is>
       </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-07-28 — Sample gauge wins; the 3-questions mock is retired; nothing to build (action item 39)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -4590,6 +4886,11 @@
           <t>Honesty gap when the network is down — the user can't tell fresh from stale. Recommend before public beta.</t>
         </is>
       </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — one banner line, still drawn for you (action item 13)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -4620,6 +4921,11 @@
           <t>The 3-day rule was your 2026-07-15 approval. Doc edit; keep the code.</t>
         </is>
       </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>DOC REFRESH — the 3-day rule was your 2026-07-15 approval; paper edit only</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -4650,6 +4956,11 @@
           <t>The per-number honesty stamps were a distinctive approved idea; unbuilt.</t>
         </is>
       </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — mock first (action item 12)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -4680,6 +4991,11 @@
           <t>Four one-line additions.</t>
         </is>
       </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — the approved banner on the other four tabs; four one-line additions</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="2" t="n">
@@ -4710,6 +5026,11 @@
           <t>One-line accessibility fix in the shared helper.</t>
         </is>
       </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 15 · your verdict pending (action item 37)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="80" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -4740,6 +5061,11 @@
           <t>The import door itself is right (you approved it post-doc) — but the wording contradiction and the landing spot need cleanup.</t>
         </is>
       </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — wording conformance on the approved doors; no new picture</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="2" t="n">
@@ -4770,6 +5096,11 @@
           <t>Three small conformance details.</t>
         </is>
       </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 14 · your verdict pending (action item 36)</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -4800,6 +5131,11 @@
           <t>Your later redesign wins. Doc edit.</t>
         </is>
       </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>DOC REFRESH — your 2026-07-15 first-run redesign wins; paper edit only</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="2" t="n">
@@ -4830,6 +5166,11 @@
           <t>Standard-expectation gap; small build.</t>
         </is>
       </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — standard pull-to-refresh gesture; the spinner is the phone’s own, no new picture</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="64" customHeight="1">
       <c r="A14" s="2" t="n">
@@ -4860,6 +5201,11 @@
           <t>A mock-approved element missing from the screen it was approved for. Decide: build the toggle or simplify the mock.</t>
         </is>
       </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 8 · picture already approved, networth-v7 FINAL (action item 9)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="2" t="n">
@@ -4890,6 +5236,11 @@
           <t>Provenance-at-a-glance was a core FCC trust idea. Recommend building on the member rows.</t>
         </is>
       </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — mock first (action item 10)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="2" t="n">
@@ -4920,6 +5271,11 @@
           <t>Approved twice (doc + final mock), never built. High-visibility gap.</t>
         </is>
       </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 7 · picture already approved, networth-v7 FINAL (action item 8)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="2" t="n">
@@ -4950,6 +5306,11 @@
           <t>Doc says yes, your final mock dropped it. Say keep-dropped (doc edit + dead code removed) or build it.</t>
         </is>
       </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-07-28 — BUILD; the Net worth screen is mocked with the cushion card first, mock batch 1 (action item 44)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="64" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -4980,6 +5341,11 @@
           <t>Plaid→SnapTrade is a doc edit. But keep-vs-delete on disconnect is a real product promise difference — pick the promise, then copy and behavior align.</t>
         </is>
       </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-07-28 + DOC REFRESH — disconnect offers the choice (copy = walk row 16); Plaid→SnapTrade is a paper edit</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="2" t="n">
@@ -5010,6 +5376,11 @@
           <t>The richer matching prevents duplicate-account messes at scale. Fine for beta; build before broad launch.</t>
         </is>
       </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — richer duplicate matching; invisible logic (action item 23)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -5040,6 +5411,11 @@
           <t>Works by accident of labeling; the explicit kind is sturdier.</t>
         </is>
       </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — one extra chip, next mock batch (action item 24)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="64" customHeight="1">
       <c r="A21" s="2" t="n">
@@ -5070,6 +5446,11 @@
           <t>The audit-trail promise ("all classes write one ledger") is broken for two asset classes. Recommend prioritizing — it is also why matured/sold money can drift unexplained.</t>
         </is>
       </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 4 · your verdict pending (action item 4)</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="80" customHeight="1">
       <c r="A22" s="2" t="n">
@@ -5100,6 +5481,11 @@
           <t>Add the same control to account detail (or a pointer to Settings), and align the wording with whichever disconnect promise you pick (see consent row).</t>
         </is>
       </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — micro-mock first; wording now decided: offer the choice (action item 22)</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="2" t="n">
@@ -5130,6 +5516,11 @@
           <t>The stamp exists at 3 of the 5 places it should. Finish the sweep.</t>
         </is>
       </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — finish the value-as-of sweep (2 of 5 places missing); tiny conformance</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="80" customHeight="1">
       <c r="A24" s="2" t="n">
@@ -5158,6 +5549,11 @@
       <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Also: at least 6 founder-approved deviations live only as code comments, never logged in the doc's Changelog tab — that is WHY the doc and app keep diverging. Recommend: every approval gets a changelog row, same day.</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>— context/coverage row · nothing to build</t>
         </is>
       </c>
     </row>
@@ -5172,7 +5568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5181,6 +5577,7 @@
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5214,6 +5611,11 @@
           <t>What it means for you / recommended action</t>
         </is>
       </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Build status — proposed vs built (added 2026-07-29; kept current)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="80" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -5244,6 +5646,11 @@
           <t>Remaining gated pieces: Fidelity application, plan upgrade before beta, Teller/banks for checking-account coverage.</t>
         </is>
       </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>DELIVERED — live and verified; remaining founder-gated: Fidelity application, plan upgrade before beta</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -5274,6 +5681,11 @@
           <t>The in-app copy is honest. Make sure marketing copy matches the same honest framing, never "we never see your data."</t>
         </is>
       </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>DELIVERED — in-app copy is honest; keep marketing copy to the same standard (your side, when written)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -5304,6 +5716,11 @@
           <t>The core hook rides an endpoint that can break without notice. The price-provider decision is the highest-leverage open external.</t>
         </is>
       </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-07-28 — I research + shortlist licensed providers; one-page recommendation coming (action item 42)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -5334,6 +5751,11 @@
           <t>Keep them (extra value, review burden) or hide them for launch (focus, less to test). 97-row sign-off includes them either way — your call.</t>
         </is>
       </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED 2026-07-28 — keep in v1; the five modules stay in your 97-row sign-off walk (action item 41)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -5364,6 +5786,11 @@
           <t>Values agree today because the copies match. One edit to one copy breaks your one-number rule silently. Extract the helper + agreement pin.</t>
         </is>
       </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 5 · your verdict pending (action item 5)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -5394,6 +5821,11 @@
           <t>Same one-number risk. Either wire the helper or delete it — an orphaned duplicate concept is a trap.</t>
         </is>
       </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — wire the shared Roth helper (one-number rule); invisible</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -5424,6 +5856,11 @@
           <t>Consolidate to one before they drift.</t>
         </is>
       </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — consolidate to one savings-capacity helper; invisible</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="2" t="n">
@@ -5454,6 +5891,11 @@
           <t>Consolidation candidate — becomes urgent when the adoption sheet is upgraded (see Plan tab).</t>
         </is>
       </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>PARKED — rides the adoption-sheet rebuild (action item 7)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -5484,6 +5926,11 @@
           <t>Same fix class as the estimate chip: one component, one wording.</t>
         </is>
       </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — one shared chip component behind the scenes; the on-row look = action item 10 (parked)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="2" t="n">
@@ -5514,6 +5961,11 @@
           <t>Minor divergence risk between the RMD table and other projections; align when touched next.</t>
         </is>
       </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — align the schedule to the shared projection engine; invisible</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="64" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -5542,6 +5994,11 @@
       <c r="F12" s="2" t="inlineStr">
         <is>
           <t>The one-concept-one-helper rule holds on 78 of 98 rows; the exceptions above are the complete list.</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>— context/coverage row · nothing to build</t>
         </is>
       </c>
     </row>
@@ -5556,7 +6013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5565,6 +6022,7 @@
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5598,6 +6056,11 @@
           <t>What it means for you / recommended action</t>
         </is>
       </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Build status — proposed vs built (added 2026-07-29; kept current)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="160" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -5628,6 +6091,11 @@
           <t>The PRD massively UNDERSTATES the product. One refresh pass brings it true. The rows below are the only genuine code-side differences that survived verification.</t>
         </is>
       </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>DOC REFRESH — one pass updates the 73 built rows; nothing to build</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="112" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -5658,6 +6126,11 @@
           <t>Adopt claim-at-62 and the hub's odds come out quietly HIGHER than the number you chose from — an optimistic cross-screen disagreement in the flagship figure. Recommend fixing before Build 46; one-line engine change + an agreement pin.</t>
         </is>
       </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 1 · accuracy · your verdict pending (action item 1)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="64" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -5688,6 +6161,11 @@
           <t>Doc edit; the two-surface agreement is intact.</t>
         </is>
       </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>DOC REFRESH — the top-bar chip was removed in an approved redesign; paper edit only</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="80" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -5718,6 +6196,11 @@
           <t>A user with vesting stock sees different month shapes on different screens. Finish the landing-month unification for equity.</t>
         </is>
       </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 6 · your verdict pending (action item 6)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -5748,6 +6231,11 @@
           <t>Known duality, still open. Consolidate when the snapshot is next touched.</t>
         </is>
       </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — consolidate the two expected-return figures; invisible</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="64" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -5778,6 +6266,11 @@
           <t>Small hole in your mask-everything rule; two-line fix.</t>
         </is>
       </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build 46 · walk row 3 · your verdict pending (action item 3)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -5808,6 +6301,11 @@
           <t>Confirm the extra gate is wanted; otherwise remove it.</t>
         </is>
       </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>OPEN — quick call: keep the extra gate (the nudge stays quiet more often) or remove it (fires whenever the plan is incomplete)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="2" t="n">
@@ -5838,6 +6336,11 @@
           <t>Wire the same taken check into the card.</t>
         </is>
       </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — wire the taken-vs-due check into the Insights card; invisible</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -5868,6 +6371,11 @@
           <t>Duplicate detection and manual-entry coverage are the two missing slices; fine for beta, note for later.</t>
         </is>
       </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — duplicate + manual-entry flag slices; invisible</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="2" t="n">
@@ -5898,6 +6406,11 @@
           <t>Accept the composed shape; doc edit.</t>
         </is>
       </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>DOC REFRESH — accept the composed engine shape; paper edit only</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -5928,6 +6441,11 @@
           <t>Post-launch cleanup with the planned legacy-migration removal.</t>
         </is>
       </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>POST-LAUNCH — rides the planned legacy-migration removal (pre-approved deferral)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="2" t="n">
@@ -5958,6 +6476,11 @@
           <t>Belongs on a device check with a legacy account, or accept the mount-time migration as the mechanism.</t>
         </is>
       </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>DEVICE CHECK — verify with a legacy account on your device walk (or accept the mount-time migration)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="2" t="n">
@@ -5988,6 +6511,11 @@
           <t>Small honest gap; either wire the real limit or label it.</t>
         </is>
       </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>NEXT WALK ROUND — wire the real HSA limit or label the zero honestly; tiny</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="2" t="n">
@@ -6016,6 +6544,11 @@
       <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Every difference that survived verification is listed above; everything else agrees.</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>— context/coverage row · nothing to build</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master file: 30 built rows → riding Build 46 (cut, #46) + 'Build 47 — plan' tab (6 ordered phases)
Build 46 note: EAS build FINISHED server-side; the CLI died with the session so
auto-submit never fired (0 submissions on the finished build) — resubmitted via
eas submit --latest, scheduled OK. Lesson: auto-submit is CLI-driven, verify
submissions on the build, not the CLI exit.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Design — Home·Net worth" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Strategy &amp; data lineage" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="PRD v1.1" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Build 47 — plan" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,8 +76,20 @@
       <color rgb="0044546A"/>
       <sz val="10.5"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -93,6 +106,11 @@
         <fgColor rgb="FFF4EAD8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B2A4A"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -106,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -138,6 +156,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1011,7 +1038,7 @@
       </c>
       <c r="H3" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1078,7 @@
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1118,7 @@
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1171,7 @@
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1211,7 @@
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1251,7 @@
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1344,7 @@
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1384,7 @@
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -2250,7 +2277,7 @@
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -2330,7 +2357,7 @@
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2397,7 @@
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -2410,7 +2437,7 @@
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -2450,7 +2477,7 @@
       </c>
       <c r="H41" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2517,7 @@
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3045,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -3193,7 +3220,7 @@
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3325,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -3473,7 +3500,7 @@
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -3673,7 +3700,7 @@
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -4233,7 +4260,7 @@
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -4783,7 +4810,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5055,7 @@
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -5098,7 +5125,7 @@
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -5203,7 +5230,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -5273,7 +5300,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5475,7 @@
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -5788,7 +5815,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -6128,7 +6155,7 @@
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -6198,7 +6225,7 @@
       </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -6268,7 +6295,7 @@
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
-          <t>BUILT — Build 46 payload (2026-07-29) · pinned by tests · suite 1,289 green</t>
+          <t>BUILT — riding Build 46 (v1.1.0 #46, CUT 2026-07-29) · pinned by tests · walk it on TestFlight</t>
         </is>
       </c>
     </row>
@@ -6549,6 +6576,204 @@
       <c r="G15" s="9" t="inlineStr">
         <is>
           <t>— context/coverage row · nothing to build</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Order</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>Which items (this file)</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>How it gets approved / what you will see</t>
+        </is>
+      </c>
+      <c r="E1" s="13" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="78" customHeight="1">
+      <c r="A2" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Your Build-46 device walk</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>Whatever you find — five suggested first checks: Net worth path-ahead row + grouping pills, Social-Security odds agreement, base-salary pop-up typing, bond partial-sale activity row, VoiceOver saying "hidden"</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>Findings go in the feedback workbook as always; fixes are always the FIRST thing in the next batch</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>WAITING ON THE BUILD — then you</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="78" customHeight="1">
+      <c r="A3" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>Mock batch 1 (pictures for approval)</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>Cushion card on Net worth (item 44) · recolored chart palettes (item 43) · first parked micro-mocks: source chips (10), staleness stamps (12), loading/offline banner (13), matured-bond banner (18)</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>Full-screen pictures per the mock rules (rich + empty states, numbers add up); each picture you approve joins Build 47, each you reject gets a doc changelog row</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>IN PROGRESS — on me now</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="78" customHeight="1">
+      <c r="A4" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Build-47 walk (no new pictures needed)</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>The ~20 NEXT WALK ROUND rows across the five tabs — e.g. Social-Security ages 67-69 state (14), Roth banner + save (16), reduce-motion (21), richer duplicate matching (23), undated-value nudge (25), hidden-balances banner on all tabs, pull-to-refresh, value-as-of sweep, the invisible helper consolidations, HSA limit</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Same as last time: one workbook, one row per fix with exact before → after, APPROVE/CHANGE/SKIP dropdowns; only approved rows build</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>NEXT — after mock batch 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="78" customHeight="1">
+      <c r="A5" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Price provider</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Item 42 — unblocks dividends &amp; total return, live pricing for thinly-traded holdings (kills the $0 class for good)</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>One-page comparison of licensed providers (coverage, dividend data, price, license terms) with a recommendation; wiring builds after your pick</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>IN PROGRESS — on me now</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="78" customHeight="1">
+      <c r="A6" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Your five open picks, brought drawn</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Debts tab month-travel (26) · cash-flow month bars (UX 6) · donut slice labels (UX 7) · winners table depth (Design 1) · plan-incomplete nudge gate (PRD 7)</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>The visual four arrive as drawn pairs in mock batches — you point at the one you want; the nudge gate you can answer any time in one sentence</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>WAITING ON YOU — no rush, none block Build 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="78" customHeight="1">
+      <c r="A7" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Cut Build 47</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Everything approved above that is built, tested and green</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>Hard gates re-run fresh (full suite, type check, clean pushed tree) → checklist presented → ships ONLY on your literal "cut the build". Quota resets Aug 1 (15 iOS builds)</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>GATED — founder word only</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build-47 phases 2+4 DELIVERED: mock batch 1 (6 hi-fi mocks, new subfolder) + price-provider one-pager
mockups/build47-batch1/ — v7 visual language, founder's real data state ($201,500,
two E*TRADE accounts), numbers add up, rich+empty states each:
cushion card (3 states) · validated palettes today-vs-proposed w/ exact hexes ·
source chips · staleness stamps (stale/fresh) · loading+offline Home · matured-bond
banner (matured/before). Nothing builds until each picture is approved.

price-provider-onepager-v1: self-serve display-license trap verified (Twelve Data
individual = no commercial display, quoted); two priced routes — Intrinio delayed
SIP ~$250/mo w/ display license (RECOMMENDED) vs Twelve Data Venture $414/mo
published (fallback); founder's 2-minute quote email included; $250-500/mo guardrail.

Master file: 15 status cells (Examples + doc tabs) -> MOCKED/DELIVERED · plan tab
phases 2+4 marked delivered.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1422,9 +1422,9 @@
           <t>PARKED — mock first, then your call.</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>PARKED — mock first · mock batch</t>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval · mockups/build47-batch1/networth-source-chips-v1-2026-07-29.html</t>
         </is>
       </c>
     </row>
@@ -1502,9 +1502,9 @@
           <t>PARKED — mock first.</t>
         </is>
       </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>PARKED — mock first · mock batch</t>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval · mockups/build47-batch1/staleness-stamps-v1-2026-07-29.html (stale vs fresh)</t>
         </is>
       </c>
     </row>
@@ -1542,9 +1542,9 @@
           <t>PARKED — mock first (it is one banner line, but you will see it drawn).</t>
         </is>
       </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>PARKED — mock first · mock batch (one banner line, still drawn for you)</t>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval · mockups/build47-batch1/home-loading-offline-v1-2026-07-29.html (offline + first-load)</t>
         </is>
       </c>
     </row>
@@ -1742,9 +1742,9 @@
           <t>PARKED — mock first (one banner).</t>
         </is>
       </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>PARKED — mock first · mock batch (one banner)</t>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval · mockups/build47-batch1/matured-bond-banner-v1-2026-07-29.html (matured vs before)</t>
         </is>
       </c>
     </row>
@@ -2728,9 +2728,9 @@
           <t>Engine only; unblocks dividends/total-return and live LCTX pricing (kills the $0 class for good).</t>
         </is>
       </c>
-      <c r="H48" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED 2026-07-28 — I research + shortlist licensed providers · one-page recommendation coming; wiring builds after your pick</t>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>ONE-PAGER DELIVERED — awaiting your pick · docs/FCC-core-55-70/price-provider-onepager-v1-2026-07-29.xlsx (recommend Intrinio, fallback Twelve Data Venture; your 2-minute email inside)</t>
         </is>
       </c>
     </row>
@@ -2768,9 +2768,9 @@
           <t>If you want the validated palettes: recolored mocks first.</t>
         </is>
       </c>
-      <c r="H49" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED 2026-07-28 — adopt the validated palettes · recolored mocks first (mock batch); builds after you approve the pictures</t>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval · mockups/build47-batch1/chart-palettes-v1-2026-07-29.html (today vs validated, exact values)</t>
         </is>
       </c>
     </row>
@@ -2808,9 +2808,9 @@
           <t>Say "drop" (doc edit + dead code removed) or "build" (mock first).</t>
         </is>
       </c>
-      <c r="H50" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED 2026-07-28 — BUILD · Net worth screen mocked with the cushion card first (mock batch 1)</t>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval · mockups/build47-batch1/networth-cushion-card-v1-2026-07-29.html (3 data states)</t>
         </is>
       </c>
     </row>
@@ -2903,9 +2903,9 @@
           <t>The app is colorblind-safe in practice (word + icon everywhere), but the palette you validated was never adopted. Decide: adopt the doc palette, or bless the shipped one and update the doc.</t>
         </is>
       </c>
-      <c r="G2" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED 2026-07-28 — adopt the validated palettes; recolored mocks first (action item 43)</t>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval · mockups/build47-batch1/chart-palettes-v1-2026-07-29.html (today vs validated, exact values)</t>
         </is>
       </c>
     </row>
@@ -2938,9 +2938,9 @@
           <t>Same-class-same-color everywhere is the point of a fixed palette. Recommend unifying on ONE keyed palette (either set) — small change, real consistency win.</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED 2026-07-28 — adopt the validated palettes; recolored mocks first (action item 43)</t>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval · mockups/build47-batch1/chart-palettes-v1-2026-07-29.html (today vs validated, exact values)</t>
         </is>
       </c>
     </row>
@@ -3908,9 +3908,9 @@
           <t>Matters for CD-heavy users; the money sits mislabeled after maturity.</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>PARKED — mock first, one banner (action item 18)</t>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval · mockups/build47-batch1/matured-bond-banner-v1-2026-07-29.html (matured vs before)</t>
         </is>
       </c>
     </row>
@@ -4913,9 +4913,9 @@
           <t>Honesty gap when the network is down — the user can't tell fresh from stale. Recommend before public beta.</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>PARKED — one banner line, still drawn for you (action item 13)</t>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval · mockups/build47-batch1/home-loading-offline-v1-2026-07-29.html (offline + first-load)</t>
         </is>
       </c>
     </row>
@@ -4983,9 +4983,9 @@
           <t>The per-number honesty stamps were a distinctive approved idea; unbuilt.</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>PARKED — mock first (action item 12)</t>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval · mockups/build47-batch1/staleness-stamps-v1-2026-07-29.html (stale vs fresh)</t>
         </is>
       </c>
     </row>
@@ -5263,9 +5263,9 @@
           <t>Provenance-at-a-glance was a core FCC trust idea. Recommend building on the member rows.</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>PARKED — mock first (action item 10)</t>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval · mockups/build47-batch1/networth-source-chips-v1-2026-07-29.html</t>
         </is>
       </c>
     </row>
@@ -5333,9 +5333,9 @@
           <t>Doc says yes, your final mock dropped it. Say keep-dropped (doc edit + dead code removed) or build it.</t>
         </is>
       </c>
-      <c r="G17" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED 2026-07-28 — BUILD; the Net worth screen is mocked with the cushion card first, mock batch 1 (action item 44)</t>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval · mockups/build47-batch1/networth-cushion-card-v1-2026-07-29.html (3 data states)</t>
         </is>
       </c>
     </row>
@@ -5743,9 +5743,9 @@
           <t>The core hook rides an endpoint that can break without notice. The price-provider decision is the highest-leverage open external.</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED 2026-07-28 — I research + shortlist licensed providers; one-page recommendation coming (action item 42)</t>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>ONE-PAGER DELIVERED — awaiting your pick · docs/FCC-core-55-70/price-provider-onepager-v1-2026-07-29.xlsx (recommend Intrinio, fallback Twelve Data Venture; your 2-minute email inside)</t>
         </is>
       </c>
     </row>
@@ -6673,7 +6673,7 @@
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>IN PROGRESS — on me now</t>
+          <t>DELIVERED 2026-07-29 — 6 mocks in mockups/build47-batch1/ · awaiting your verdicts</t>
         </is>
       </c>
     </row>
@@ -6723,7 +6723,7 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>IN PROGRESS — on me now</t>
+          <t>DELIVERED 2026-07-29 — one-pager in docs/FCC-core-55-70/ · awaiting your pick</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build-47 walk workbook delivered: 21 no-picture rows (honesty/consolidation/conformance/accessibility) + 27 master-file cells -> PROPOSED
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1582,9 +1582,9 @@
           <t>Same approved table, different rows for this age group. I will include the 68-year-old state in the next mock batch for your eyes.</t>
         </is>
       </c>
-      <c r="H18" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — approved table pattern, no new picture; I will propose it with the 68-year-old state included</t>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 2 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -1662,9 +1662,9 @@
           <t>The banner = the exact approved element from sibling screens (conforming). The hub action item is new — mock first for that part.</t>
         </is>
       </c>
-      <c r="H20" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — conforming banner (approved element from sibling screens) + the hub action item</t>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 15 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -1862,9 +1862,9 @@
           <t>Nothing changes for you — only for users who asked their phone for less motion.</t>
         </is>
       </c>
-      <c r="H25" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — invisible (respects the phone’s reduce-motion setting); no picture needed</t>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 20 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -1942,9 +1942,9 @@
           <t>Invisible logic — just fewer duplicate-account accidents.</t>
         </is>
       </c>
-      <c r="H27" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — invisible logic; no picture needed</t>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk (folded into row 19) · verdict pending</t>
         </is>
       </c>
     </row>
@@ -2022,9 +2022,9 @@
           <t>One line in the approved nudge style.</t>
         </is>
       </c>
-      <c r="H29" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — one line in the approved nudge style</t>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 5 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -3008,9 +3008,9 @@
           <t>Visual drift risk, not a correctness bug. Worth one consolidation pass after launch-critical work.</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — one shared hero component at today’s sizes; invisible consolidation</t>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 11 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -3428,9 +3428,9 @@
           <t>Screen-reader coverage is real but ad-hoc. Either add the label to the shared component or re-word the doc rule to match the per-card pattern.</t>
         </is>
       </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — spoken label on the shared money component + a guard test; invisible</t>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 21 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -3463,9 +3463,9 @@
           <t>Real accessibility gap for a 65+ audience. Moderate effort; recommend post-Build-46 but before public launch.</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — respects the phone’s reduce-motion setting; invisible (action item 21)</t>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 20 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -3838,9 +3838,9 @@
           <t>Mild but confusing when you switch periods. Small fix.</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — detail mirrors the selected period; small conformance, no new picture</t>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 16 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -3873,9 +3873,9 @@
           <t>Small reach-through interaction never wired.</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — tap scrolls to the holding; small interaction, no new picture</t>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 17 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -4398,9 +4398,9 @@
           <t>Real cohort in your 55-70 target. Recommend fixing.</t>
         </is>
       </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — approved table pattern incl. the 68-year-old state; no new picture (action item 14)</t>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 2 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -4468,9 +4468,9 @@
           <t>The banner is also a UX-doc rule; the action item is the follow-through that makes adoption real.</t>
         </is>
       </c>
-      <c r="G25" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — conforming banner + save + dated action item (action item 16)</t>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 15 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -4608,9 +4608,9 @@
           <t>One-line suppression rule.</t>
         </is>
       </c>
-      <c r="G29" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — one-line suppression rule; invisible</t>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 18 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -4643,9 +4643,9 @@
           <t>Quiet data-quality hole; small fix.</t>
         </is>
       </c>
-      <c r="G30" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — one line in the approved nudge style (action item 25)</t>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 5 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -5018,9 +5018,9 @@
           <t>Four one-line additions.</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — the approved banner on the other four tabs; four one-line additions</t>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 12 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -5088,9 +5088,9 @@
           <t>The import door itself is right (you approved it post-doc) — but the wording contradiction and the landing spot need cleanup.</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — wording conformance on the approved doors; no new picture</t>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 14 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -5193,9 +5193,9 @@
           <t>Standard-expectation gap; small build.</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — standard pull-to-refresh gesture; the spinner is the phone’s own, no new picture</t>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 13 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -5403,9 +5403,9 @@
           <t>The richer matching prevents duplicate-account messes at scale. Fine for beta; build before broad launch.</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — richer duplicate matching; invisible logic (action item 23)</t>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk (richer duplicate matching folded into row 19's flag work) · verdict pending</t>
         </is>
       </c>
     </row>
@@ -5543,9 +5543,9 @@
           <t>The stamp exists at 3 of the 5 places it should. Finish the sweep.</t>
         </is>
       </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — finish the value-as-of sweep (2 of 5 places missing); tiny conformance</t>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 4 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -5848,9 +5848,9 @@
           <t>Same one-number risk. Either wire the helper or delete it — an orphaned duplicate concept is a trap.</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — wire the shared Roth helper (one-number rule); invisible</t>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 6 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -5883,9 +5883,9 @@
           <t>Consolidate to one before they drift.</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — consolidate to one savings-capacity helper; invisible</t>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 7 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -5953,9 +5953,9 @@
           <t>Same fix class as the estimate chip: one component, one wording.</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — one shared chip component behind the scenes; the on-row look = action item 10 (parked)</t>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 8 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -5988,9 +5988,9 @@
           <t>Minor divergence risk between the RMD table and other projections; align when touched next.</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — align the schedule to the shared projection engine; invisible</t>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 9 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -6258,9 +6258,9 @@
           <t>Known duality, still open. Consolidate when the snapshot is next touched.</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — consolidate the two expected-return figures; invisible</t>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 10 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -6363,9 +6363,9 @@
           <t>Wire the same taken check into the card.</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — wire the taken-vs-due check into the Insights card; invisible</t>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 3 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -6398,9 +6398,9 @@
           <t>Duplicate detection and manual-entry coverage are the two missing slices; fine for beta, note for later.</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — duplicate + manual-entry flag slices; invisible</t>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 19 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -6538,9 +6538,9 @@
           <t>Small honest gap; either wire the real limit or label it.</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>NEXT WALK ROUND — wire the real HSA limit or label the zero honestly; tiny</t>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>PROPOSED — Build-47 walk row 1 · your verdict pending (build47-item-walk-v1-2026-07-29.xlsx)</t>
         </is>
       </c>
     </row>
@@ -6698,7 +6698,7 @@
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>NEXT — after mock batch 1</t>
+          <t>DELIVERED 2026-07-29 — build47-item-walk-v1-2026-07-29.xlsx (21 rows) · awaiting your verdicts</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
One master file (founder order): Build-46 findings become a tab in build-analysis-july24.xlsx; separate feedback workbook retired
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -8,13 +8,14 @@
   <sheets>
     <sheet name="How to read" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="SUMMARY — read me first" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Examples &amp; mock map" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="UX design v1.1" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Design — Invest·CF·Plan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Design — Home·Net worth" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Strategy &amp; data lineage" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="PRD v1.1" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Build 47 — plan" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Build 46 — findings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Examples &amp; mock map" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="UX design v1.1" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Design — Invest·CF·Plan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Design — Home·Net worth" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Strategy &amp; data lineage" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="PRD v1.1" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Build 47 — plan" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -112,7 +113,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -120,11 +121,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9D2E0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C9D2E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9D2E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9D2E0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -165,6 +180,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -532,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -596,6 +620,216 @@
       <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Your one-master-file request: EVERY tab now carries a Build status column (H on Examples &amp; mock map, G on the five document tabs). It says for each row: PROPOSED for Build 46 (with its row in the walk workbook) · PARKED at the mock gate · NEXT WALK ROUND (no picture needed, proposed after this batch) · DECIDED (your call, dated) · OPEN (a pick still yours to make) · DOC REFRESH (paper edit only, nothing to build) · DELIVERED · NO ACTION (deliberate, founder-known deviation) · DEVICE CHECK · POST-LAUNCH. Rows that map to an action item cite it, so the tabs can never disagree. As items build I update the cells to "BUILT — Build N" the same day. This file is the master monitor; build46-item-walk-v1-2026-07-28.xlsx is just the approval form for the current batch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="56" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Build 46 — findings tab (added 2026-07-29)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Your device-walk findings for Build 46 live HERE (one master file, your standing rule) — numbered rows with what you saw, the verified root cause, the fix and its status. I add rows as your findings arrive and update statuses the same day fixes build. The old separate feedback workbook is retired; future builds get their own findings tab the same way.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Order</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>Which items (this file)</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>How it gets approved / what you will see</t>
+        </is>
+      </c>
+      <c r="E1" s="13" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="78" customHeight="1">
+      <c r="A2" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Your Build-46 device walk</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>Whatever you find — five suggested first checks: Net worth path-ahead row + grouping pills, Social-Security odds agreement, base-salary pop-up typing, bond partial-sale activity row, VoiceOver saying "hidden"</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>Findings go in the feedback workbook as always; fixes are always the FIRST thing in the next batch</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>WAITING ON THE BUILD — then you</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="78" customHeight="1">
+      <c r="A3" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>Mock batch 1 (pictures for approval)</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>Cushion card on Net worth (item 44) · recolored chart palettes (item 43) · first parked micro-mocks: source chips (10), staleness stamps (12), loading/offline banner (13), matured-bond banner (18)</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>Full-screen pictures per the mock rules (rich + empty states, numbers add up); each picture you approve joins Build 47, each you reject gets a doc changelog row</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>DELIVERED 2026-07-29 — 6 mocks in mockups/build47-batch1/ · awaiting your verdicts</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="78" customHeight="1">
+      <c r="A4" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Build-47 walk (no new pictures needed)</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>The ~20 NEXT WALK ROUND rows across the five tabs — e.g. Social-Security ages 67-69 state (14), Roth banner + save (16), reduce-motion (21), richer duplicate matching (23), undated-value nudge (25), hidden-balances banner on all tabs, pull-to-refresh, value-as-of sweep, the invisible helper consolidations, HSA limit</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Same as last time: one workbook, one row per fix with exact before → after, APPROVE/CHANGE/SKIP dropdowns; only approved rows build</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>DELIVERED 2026-07-29 — build47-item-walk-v1-2026-07-29.xlsx (21 rows) · awaiting your verdicts</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="78" customHeight="1">
+      <c r="A5" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Price provider</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Item 42 — unblocks dividends &amp; total return, live pricing for thinly-traded holdings (kills the $0 class for good)</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>One-page comparison of licensed providers (coverage, dividend data, price, license terms) with a recommendation; wiring builds after your pick</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>DELIVERED 2026-07-29 — one-pager in docs/FCC-core-55-70/ · awaiting your pick</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="78" customHeight="1">
+      <c r="A6" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Your five open picks, brought drawn</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Debts tab month-travel (26) · cash-flow month bars (UX 6) · donut slice labels (UX 7) · winners table depth (Design 1) · plan-incomplete nudge gate (PRD 7)</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>The visual four arrive as drawn pairs in mock batches — you point at the one you want; the nudge gate you can answer any time in one sentence</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>WAITING ON YOU — no rush, none block Build 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="78" customHeight="1">
+      <c r="A7" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Cut Build 47</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Everything approved above that is built, tested and green</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>Hard gates re-run fresh (full suite, type check, clean pushed tree) → checklist presented → ships ONLY on your literal "cut the build". Quota resets Aug 1 (15 iOS builds)</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>GATED — founder word only</t>
         </is>
       </c>
     </row>
@@ -934,6 +1168,154 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>What you saw</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>Verified root cause</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>The fix</t>
+        </is>
+      </c>
+      <c r="E1" s="13" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="118" customHeight="1">
+      <c r="A2" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>Q: does import bring in dividends &amp; interest?</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>Not a bug — answered: connected accounts import dividends/interest/coupons into the account Activity, the income surfaces and the tax estimate; Invest returns stay price-only until the price provider lands; the file import brings holdings only.</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>No fix needed. The "Dividends &amp; interest" line on Cash flow This-month is audit item 27 (parked, mock on request).</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>ANSWERED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="118" customHeight="1">
+      <c r="A3" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Look-ahead sliders still frozen on Build 46 (second failed fix)</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>TWO device-only causes my simulated-touch tests could not see: (a) the screen's scroll view NATIVELY cancels the drag after a few points — refusing the termination request does not stop iOS; (b) the mid-drag touch coordinate is read relative to whatever sits under the finger and goes stale off the strip.</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>Slider rebuilt: claims the touch at capture, the scroll view is disabled while a finger is down (new handshake, pinned), and every move is driven by page-absolute coordinates anchored at touch-down. 11 pins incl. the scroll-stand-down behavior. RIDES BUILD 47 — device verification is yours; I will not call it fixed until your thumb says so.</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>FIX BUILT — verify on 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="118" customHeight="1">
+      <c r="A4" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Add investment: picking Bonds / Crypto / Private equity / Hedge funds never changes the form; an added option landed under Stocks/ETFs</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>The sheet offers all 8 investment types as chips but the chips only switch the BENCHMARK — the form is ticker/shares/cost for everything. Verified root cause of the option case: this sheet always creates a ticker POSITION, and positions can only render in the equities bucket (options/alternatives are value-based ACCOUNTS in our model, added on their own editors with the right forms). Per the master file this screen is "complete" — the docs never asked it to adapt, which is exactly the gap your walk found: a document blind spot, not code drift.</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>PROPOSED: the type chips become a router — Stocks/ETFs keep the ticker form; Fixed income routes to the bond editor (face/coupon/maturity); Options/Crypto/Private equity/Hedge funds/Gold route to the alternatives editor pre-set to that type. Sheet change → per your mock-first rule I mock it before building (joining the mock batch under review).</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>OPEN — mock next</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="118" customHeight="1">
+      <c r="A5" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Record-a-transaction: the account picker shows "E*Trade savings" three times + "E*Trade brokerage" once — you only uploaded one account</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>VERIFIED: your statement upload deliberately splits by type — LCTX became a brokerage account, and every CASH-type line on the file (money market / sweep / CD-like rows) became its OWN small account, each filed under Cash with institution E*Trade. Three cash lines → three accounts. The picker then names chips its own local way (institution first; on a name collision it appends the TYPE) instead of the shared account-naming helper the rest of the app uses — three accounts sharing institution AND type = three IDENTICAL chips. A one-concept-one-helper violation (same class as your B43 finding 9).</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Fix (a): the picker adopts the shared account naming — you would see the real names (e.g. the fund name, "· 1 / · 2") instead of three clones. Proposed as Build-47 walk row 22 (conforms to the approved naming system, no new design). Check (b) FOR YOU: those three accounts may DOUBLE-COUNT money your live E*TRADE connection already reports — open Net worth → the Cash class (or the new By-institution pill) and look at their names and amounts; if they duplicate connected money, they should be deleted. Tell me what you see and I will guide or script the cleanup.</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>FIX PROPOSED + your 30-sec check</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
@@ -2819,7 +3201,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3579,7 +3961,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4724,7 +5106,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5589,7 +5971,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6034,7 +6416,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6582,202 +6964,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="13" t="inlineStr">
-        <is>
-          <t>Order</t>
-        </is>
-      </c>
-      <c r="B1" s="13" t="inlineStr">
-        <is>
-          <t>What</t>
-        </is>
-      </c>
-      <c r="C1" s="13" t="inlineStr">
-        <is>
-          <t>Which items (this file)</t>
-        </is>
-      </c>
-      <c r="D1" s="13" t="inlineStr">
-        <is>
-          <t>How it gets approved / what you will see</t>
-        </is>
-      </c>
-      <c r="E1" s="13" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="78" customHeight="1">
-      <c r="A2" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="15" t="inlineStr">
-        <is>
-          <t>Your Build-46 device walk</t>
-        </is>
-      </c>
-      <c r="C2" s="15" t="inlineStr">
-        <is>
-          <t>Whatever you find — five suggested first checks: Net worth path-ahead row + grouping pills, Social-Security odds agreement, base-salary pop-up typing, bond partial-sale activity row, VoiceOver saying "hidden"</t>
-        </is>
-      </c>
-      <c r="D2" s="15" t="inlineStr">
-        <is>
-          <t>Findings go in the feedback workbook as always; fixes are always the FIRST thing in the next batch</t>
-        </is>
-      </c>
-      <c r="E2" s="14" t="inlineStr">
-        <is>
-          <t>WAITING ON THE BUILD — then you</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="78" customHeight="1">
-      <c r="A3" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="15" t="inlineStr">
-        <is>
-          <t>Mock batch 1 (pictures for approval)</t>
-        </is>
-      </c>
-      <c r="C3" s="15" t="inlineStr">
-        <is>
-          <t>Cushion card on Net worth (item 44) · recolored chart palettes (item 43) · first parked micro-mocks: source chips (10), staleness stamps (12), loading/offline banner (13), matured-bond banner (18)</t>
-        </is>
-      </c>
-      <c r="D3" s="15" t="inlineStr">
-        <is>
-          <t>Full-screen pictures per the mock rules (rich + empty states, numbers add up); each picture you approve joins Build 47, each you reject gets a doc changelog row</t>
-        </is>
-      </c>
-      <c r="E3" s="14" t="inlineStr">
-        <is>
-          <t>DELIVERED 2026-07-29 — 6 mocks in mockups/build47-batch1/ · awaiting your verdicts</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="78" customHeight="1">
-      <c r="A4" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="15" t="inlineStr">
-        <is>
-          <t>Build-47 walk (no new pictures needed)</t>
-        </is>
-      </c>
-      <c r="C4" s="15" t="inlineStr">
-        <is>
-          <t>The ~20 NEXT WALK ROUND rows across the five tabs — e.g. Social-Security ages 67-69 state (14), Roth banner + save (16), reduce-motion (21), richer duplicate matching (23), undated-value nudge (25), hidden-balances banner on all tabs, pull-to-refresh, value-as-of sweep, the invisible helper consolidations, HSA limit</t>
-        </is>
-      </c>
-      <c r="D4" s="15" t="inlineStr">
-        <is>
-          <t>Same as last time: one workbook, one row per fix with exact before → after, APPROVE/CHANGE/SKIP dropdowns; only approved rows build</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>DELIVERED 2026-07-29 — build47-item-walk-v1-2026-07-29.xlsx (21 rows) · awaiting your verdicts</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="78" customHeight="1">
-      <c r="A5" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>Price provider</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>Item 42 — unblocks dividends &amp; total return, live pricing for thinly-traded holdings (kills the $0 class for good)</t>
-        </is>
-      </c>
-      <c r="D5" s="15" t="inlineStr">
-        <is>
-          <t>One-page comparison of licensed providers (coverage, dividend data, price, license terms) with a recommendation; wiring builds after your pick</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>DELIVERED 2026-07-29 — one-pager in docs/FCC-core-55-70/ · awaiting your pick</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="78" customHeight="1">
-      <c r="A6" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>Your five open picks, brought drawn</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>Debts tab month-travel (26) · cash-flow month bars (UX 6) · donut slice labels (UX 7) · winners table depth (Design 1) · plan-incomplete nudge gate (PRD 7)</t>
-        </is>
-      </c>
-      <c r="D6" s="15" t="inlineStr">
-        <is>
-          <t>The visual four arrive as drawn pairs in mock batches — you point at the one you want; the nudge gate you can answer any time in one sentence</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>WAITING ON YOU — no rush, none block Build 47</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="78" customHeight="1">
-      <c r="A7" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="15" t="inlineStr">
-        <is>
-          <t>Cut Build 47</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>Everything approved above that is built, tested and green</t>
-        </is>
-      </c>
-      <c r="D7" s="15" t="inlineStr">
-        <is>
-          <t>Hard gates re-run fresh (full suite, type check, clean pushed tree) → checklist presented → ships ONLY on your literal "cut the build". Quota resets Aug 1 (15 iOS builds)</t>
-        </is>
-      </c>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>GATED — founder word only</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
B46 finding 5: imported cash trio double-counts vs connected balances (real case for audit item 23); walk row 23 = confirm-before-remove
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1168,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1302,6 +1302,31 @@
       <c r="E5" s="18" t="inlineStr">
         <is>
           <t>FIX PROPOSED + your 30-sec check</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="128" customHeight="1">
+      <c r="A6" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>NW → Cash shows "E*Trade Key bank CD", "E*Trade VMFXX", "E*Trade cash" — leftovers from the statement upload, alongside the SAME money inside the connected accounts</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>CONFIRMED double-count risk: your connected E*TRADE accounts already report the money market + cash (the "· 2 money market + cash in this account" row) and the CDs; the connect-time merge could not absorb the imported trio because imports carry no account number to match on (the audit's "richer duplicate matching" gap, item 23 — now proven by a real case). Also observed while verifying the fix path: the editor's Remove button deletes an account IMMEDIATELY with no confirmation step.</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>For you now: remove the three imported leftovers (taps in chat). For Build 47: (a) richer duplicate matching gets elevated — connect-time merge should flag same-institution manual/imported accounts as likely twins and ask; (b) Remove gains a confirm step ("Remove E*Trade VMFXX? Its $X leaves your net worth") — joins the walk as row 23.</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>YOUR CLEANUP + 2 fixes queued</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B46 finding 5 RESOLVED by founder's broker check: no double-count — imported trio complements connected balances; keep accounts; merge fix specced ask-first
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1316,17 +1316,17 @@
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>CONFIRMED double-count risk: your connected E*TRADE accounts already report the money market + cash (the "· 2 money market + cash in this account" row) and the CDs; the connect-time merge could not absorb the imported trio because imports carry no account number to match on (the audit's "richer duplicate matching" gap, item 23 — now proven by a real case). Also observed while verifying the fix path: the editor's Remove button deletes an account IMMEDIATELY with no confirmation step.</t>
+          <t>RESOLVED BY YOUR CHECK (2026-07-29): totals MATCH the broker — NO double-count. The three imported accounts (KeyBank CD, VMFXX, cash) carry money the live connection's reported balances do NOT include — the import complements the connection. KEEP all three. Design lesson captured: the future duplicate-matching fix must ASK, never auto-absorb — auto-merging here would have silently deleted real money.</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>For you now: remove the three imported leftovers (taps in chat). For Build 47: (a) richer duplicate matching gets elevated — connect-time merge should flag same-institution manual/imported accounts as likely twins and ask; (b) Remove gains a confirm step ("Remove E*Trade VMFXX? Its $X leaves your net worth") — joins the walk as row 23.</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>YOUR CLEANUP + 2 fixes queued</t>
+          <t>No cleanup. Still queued from this finding: walk row 22 (the picker's identical "E*Trade savings" chips → shared naming) and walk row 23 (confirm before Remove). The richer duplicate-matching fix (walk row 19 scope) is now specced as ask-first.</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>RESOLVED — keep accounts</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B46 finding 6: Record-transaction sheet has no bond/alternative path — folded into the finding-3 router mock (one drawing, both sheets)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1168,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1327,6 +1327,31 @@
       <c r="E6" s="17" t="inlineStr">
         <is>
           <t>RESOLVED — keep accounts</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="118" customHeight="1">
+      <c r="A7" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Invest → Record a transaction only supports stocks/ETFs and cash actions (Buy / Sell / Deposit / Withdraw / Transfer / Dividend) — nothing for bonds or alternatives</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>VERIFIED: deliberate in the code ("cash actions apply to equity + cash accounts — never bond or alternative accounts, those aren't traded here") — bonds and alternatives transact inside their OWN screens (the Bonds and Alternatives editors, which since Build 46 write real Sell rows to the ledger). But the central Record sheet gives NO door or pointer to those flows: a bond/CD holder standing on Invest has no path from here. Same document blind spot as finding 3 — the docs designed separate flows and never asked the central sheet to route to them.</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>ONE fix for findings 3 + 6 together: a router. On the Add sheet, type chips route to the right editor (finding 3); on the Record sheet, a "Bond / CD / alternative" path routes to that account's own record flow. Both are the same drawing — ONE mock covering both sheets joins the batch you're reviewing.</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>OPEN — mock next (with #3)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B46 finding 7: THIS-MONTH surplus = In − Out by construction (was a second engine behind an equals sign, off by $572 on device); identity pinned to the dollar
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1168,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1352,6 +1352,31 @@
       <c r="E7" s="18" t="inlineStr">
         <is>
           <t>OPEN — mock next (with #3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="120" customHeight="1">
+      <c r="A8" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Cash flow THIS MONTH: "In (take-home) $8,600 − Out (bills) $0 = Planned surplus $9,172" — the equation is false on its face; and the Income tab source says salary steady $5,000</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>VERIFIED root cause of the false equation: the In and Out lines read the month grid, but the surplus line read a DIFFERENT engine (the plan-level savings-capacity helper) whose income basis can legitimately differ — the card printed two engines with an equals sign between them. Exactly the "two savings-capacity helpers" drift the audit flagged (Strategy tab #7), now caught making the app contradict itself on one card.</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>FIXED same hour: the surplus row is now COMPUTED as In − Out from the same month cell — the equals sign is earned by construction, pinned by a test that renders the card and checks the arithmetic to the dollar. Rides Build 47. The engine-level consolidation (one capacity helper) remains walk row 7. STILL OPEN: why In shows $8,600 when your only listed source is $5,000 steady — answering needs one fact from your screen (see chat).</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>FIXED (card) — verify on 47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B46 finding 8: Income-tab salary row told a hardcoded 'take-home · monthly' story — now names the stored form and bridges to the same monthly take-home the In line uses (cross-tab pin)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1168,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1377,6 +1377,31 @@
       <c r="E8" s="17" t="inlineStr">
         <is>
           <t>FIXED (card) — verify on 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="126" customHeight="1">
+      <c r="A9" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Income tab says "Salary — steady $5,000, take-home · monthly" but the This-month In line says $8,600 — and Salary is the ONLY source</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>VERIFIED: the Salary row printed the raw per-period entry and HARDCODED the words "take-home · monthly" no matter what the stored fields say. Your stored salary is almost certainly a per-period, before-tax figure (e.g. $5,000 every 2 weeks before tax ≈ $10,833/mo gross ≈ $8,600/mo after tax) — so the In line was HONEST and the sources row was the wrong number. The income pop-up always writes monthly take-home, so this salary was captured through an older path (or an earlier cloud profile) with different units.</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>FIXED same hour: the row now names the entered form truthfully and bridges to the SAME monthly take-home the In line uses ("before tax · every 2 weeks · ≈ $8,600/mo take-home") — pinned with a cross-tab reconciliation test. Rides Build 47. FOR YOU: confirm the stored form matches reality — if your true pay IS $5,000/mo take-home, open ＋ Set up income, re-save steady $5,000, and every number follows; if it is $5,000 per paycheck before tax, the app was right all along and now says so.</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>FIXED (display) — your data check</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B46 finding 9: Income-tab note is internal jargon pointing at an unreachable place; equity/rental editors gated behind rows that only exist when already captured — walk rows 24-25
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1168,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1402,6 +1402,31 @@
       <c r="E9" s="17" t="inlineStr">
         <is>
           <t>FIXED (display) — your data check</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="126" customHeight="1">
+      <c r="A10" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Income tab note reads "Opens the steady-or-varies question. Rich editors (equity comp, rental) live in the income manager" — what does it mean, and where are these editors? Both paths show only one number</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>THREE verified problems in one note: (a) it is written in my internal jargon — "steady-or-varies question", "rich editors", "income manager" are code words, not app words (the menu calls that screen just "Income"); (b) it points somewhere without taking you there — no link; (c) the REAL bug: on the Income screen, the stock-vesting and rental editors open ONLY by tapping an existing "Equity comp" or "Rental property" row — and those rows render only when the amount is already above zero. Anyone who skipped them at onboarding has NO path to ever add them. That is why you saw one number and no doors.</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>Queued as two walk rows with exact before→after: row 24 — the note becomes plain English with a real door ("Pay from stock vesting or a rental? They have their own screen — open Income ›"); row 25 — the Income screen gains an "＋ Add an income source" path (bonus, stock vesting, rental, self-employment) so the editors are reachable for everyone, not just onboarding completers.</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>OPEN — walk rows 24-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Findings tab hygiene: finding 4 status reflects #5's resolution
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -139,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -189,6 +189,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1299,9 +1302,9 @@
           <t>Fix (a): the picker adopts the shared account naming — you would see the real names (e.g. the fund name, "· 1 / · 2") instead of three clones. Proposed as Build-47 walk row 22 (conforms to the approved naming system, no new design). Check (b) FOR YOU: those three accounts may DOUBLE-COUNT money your live E*TRADE connection already reports — open Net worth → the Cash class (or the new By-institution pill) and look at their names and amounts; if they duplicate connected money, they should be deleted. Tell me what you see and I will guide or script the cleanup.</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>FIX PROPOSED + your 30-sec check</t>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>FIX PROPOSED — walk row 22 (double-count check closed by #5: keep accounts)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Router mock delivered (findings 3+6, one drawing, both sheets) — the last open on-me Build-47 item; findings tab statuses → MOCKED
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1277,9 +1277,9 @@
           <t>PROPOSED: the type chips become a router — Stocks/ETFs keep the ticker form; Fixed income routes to the bond editor (face/coupon/maturity); Options/Crypto/Private equity/Hedge funds/Gold route to the alternatives editor pre-set to that type. Sheet change → per your mock-first rule I mock it before building (joining the mock batch under review).</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
-        <is>
-          <t>OPEN — mock next</t>
+      <c r="E4" s="19" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval · mockups/build47-batch1/invest-add-record-router-v1-2026-07-30.html</t>
         </is>
       </c>
     </row>
@@ -1352,9 +1352,9 @@
           <t>ONE fix for findings 3 + 6 together: a router. On the Add sheet, type chips route to the right editor (finding 3); on the Record sheet, a "Bond / CD / alternative" path routes to that account's own record flow. Both are the same drawing — ONE mock covering both sheets joins the batch you're reviewing.</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>OPEN — mock next (with #3)</t>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval · mockups/build47-batch1/invest-add-record-router-v1-2026-07-30.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B46 finding 10: ACME receipt $8.99/$9.99 vs true $4.99 — ranked totals (BALANCE class), savings-section decoy guard, negative-line exclusion, payment-echo fallback; founder receipt pinned in BOTH parsers
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1171,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1430,6 +1430,31 @@
       <c r="E10" s="18" t="inlineStr">
         <is>
           <t>OPEN — walk rows 24-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="132" customHeight="1">
+      <c r="A11" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Receipt scan reads the ACME receipt as $8.99 or $9.99 — the real bill was $4.99</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>VERIFIED from your photo — three traps on one slip: (a) the true total prints as "**** BALANCE", and bare "balance" was not a total keyword (only "balance due"); (b) the savings section prints a decoy "Total 4.00" (your coupons, not your bill); (c) whenever OCR mangles the keywords, the fallback took the LARGEST safe number — the $8.99 list price. $9.99 = OCR digit noise on the same wrong pick. Same parser class as your Build-44 cash-tendered finding.</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>FIXED same hour in BOTH parsers (the Build-44 lesson): ranked totals — the BALANCE/amount-due class beats a bare "total"; once a savings/points section starts, bare "Total" lines stop counting; discount lines (negative) are never charges; and a payment ECHO (an amount matching what you actually paid — $4.99 on three lines) beats the largest-number fallback, so even a keyword-mangled scan lands on $4.99. Your receipt is the pinned fixture, plus a mangled-keyword variant. Rides Build 47.</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>FIXED — verify on 47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Palette mock v2 (v1 kept): founder feedback — real approved screens only (no invented NW section), ONE explicit yes/no question; NW as Build-46 ships + Invest as its own phone, today vs proposed
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -3305,7 +3305,7 @@
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>MOCKED — awaiting your approval · mockups/build47-batch1/chart-palettes-v1-2026-07-29.html (today vs validated, exact values)</t>
+          <t>MOCKED v2 — awaiting your yes/no · mockups/build47-batch1/chart-palettes-v2-2026-07-30.html (v1 feedback applied: real screens only, one explicit question)</t>
         </is>
       </c>
     </row>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>MOCKED — awaiting your approval · mockups/build47-batch1/chart-palettes-v1-2026-07-29.html (today vs validated, exact values)</t>
+          <t>MOCKED v2 — awaiting your yes/no · mockups/build47-batch1/chart-palettes-v2-2026-07-30.html (v1 feedback applied: real screens only, one explicit question)</t>
         </is>
       </c>
     </row>
@@ -3475,7 +3475,7 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>MOCKED — awaiting your approval · mockups/build47-batch1/chart-palettes-v1-2026-07-29.html (today vs validated, exact values)</t>
+          <t>MOCKED v2 — awaiting your yes/no · mockups/build47-batch1/chart-palettes-v2-2026-07-30.html (v1 feedback applied: real screens only, one explicit question)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build 47 CUT on founder word: plan tab updated — 1,321 green, review 49/49 pinned
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -807,7 +807,7 @@
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>WAITING ON YOU — no rush, none block Build 47</t>
+          <t>ALL RESOLVED in the verdict rounds (dots C, growth link keep, periods keep) except the plan-incomplete nudge gate (PRD 7) — still open, answer any time</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>GATED — founder word only</t>
+          <t>CUT 2026-07-31 on your word ("cut build 47") — gates fresh: 1,321 green, type check clean, clean pushed tree; code-vs-master review PASSED (49 of 49 payload claims pinned); EAS building → auto-submit → TestFlight</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B47 finding 4: delete-holding exits silently (leaving guard) — the deletion was correct, the not-found flash read as an error; pinned; findings tab updated
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -2020,7 +2020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2129,6 +2129,31 @@
       <c r="E4" s="17" t="inlineStr">
         <is>
           <t>FIXED — pull to heal · verify on 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="100" customHeight="1">
+      <c r="A5" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Invest → holding detail → delete holding: an error screen shows — but the holding did get deleted</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>VERIFIED: the deletion itself was always correct. Deleting re-renders the page BEFORE the back-navigation finishes, so the "This holding isn't here any more" fallback flashed mid-exit and read as an error.</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>FIXED same hour: the delete path now exits silently — the page renders nothing during the leave, then you land back on Invest with the holding gone. The not-found screen still exists for its real case (opening a link to a holding deleted elsewhere). Rides Build 48.</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>FIXED — verify on 48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B47 findings 5+6: CD-shaped positions map to Bonds & CDs (description heuristics, look-alike-safe, pinned); holding-detail hero mocked to founder spec (price → graph → facts table)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -2020,7 +2020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2154,6 +2154,56 @@
       <c r="E5" s="17" t="inlineStr">
         <is>
           <t>FIXED — verify on 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="110" customHeight="1">
+      <c r="A6" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>A CD shows under Stocks/ETFs on the Invest screen</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>VERIFIED: only the explicit bond type code mapped to Bonds &amp; CDs — Vanguard's brokered CD arrives without it and fell through to equities (the same positions-default class as your option finding).</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>FIXED same hour: fixed-income SHAPES are recognized by description too — CDs, certificates of deposit, Treasuries/T-bills, and coupon-with-maturity patterns land in Bonds &amp; CDs (the bucket your E*TRADE CDs always used). Ticker look-alikes (MCD) are not fooled — pinned both ways. Your Vanguard heals on its next sync. Rides Build 48.</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>FIXED — pull to heal · verify on 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="110" customHeight="1">
+      <c r="A7" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Holding-detail hero: current design disliked — should be price on top, then graph, then value / change since purchase $ and % / quantity / price, in a table</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Design direction, not a bug — your spec recorded verbatim.</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>MOCKED to your exact order: mockups/build47-batch1/holding-detail-hero-v1-2026-07-31.html (real arithmetic, tabular numerals, everything below the hero untouched). Approve the picture and it builds into Build 48.</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B47 finding 7: slice-tap class-view mocked (founder direction; honest correction recorded — E*TRADE never worked that way, docs+code agree)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -2020,7 +2020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2202,6 +2202,31 @@
         </is>
       </c>
       <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="110" customHeight="1">
+      <c r="A8" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Tapping the Stocks/ETFs slice of a mixed account should land on a stocks-only view — "that's the design and how E*TRADE worked"</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>HONEST CORRECTION, verified in code and docs: it never worked that way — every slice tap opened the FULL account page, for E*TRADE too; the approved docs specify the account page. The what's-inside-by-type breakdown at the top made it FEEL class-focused. Your expectation is now the direction.</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>MOCKED: mockups/build47-batch1/account-class-view-v1-2026-07-31.html — slice tap lands on the class-only view (portion hero, that class's holdings summing visibly, whole account one tap away; account taps elsewhere unchanged). Approve and it builds into Build 48.</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
         <is>
           <t>MOCKED — awaiting your approval</t>
         </is>

</xml_diff>

<commit_message>
B47 finding 8: activity prices cents-precise (B44 rule, missed sheet) + one word Activity (button matched to sheet); pinned
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -2020,7 +2020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2229,6 +2229,31 @@
       <c r="E8" s="19" t="inlineStr">
         <is>
           <t>MOCKED — awaiting your approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="100" customHeight="1">
+      <c r="A9" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Holding detail → the history list shows sell price as an integer, not cents; and the button says History while the sheet says Activity</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>VERIFIED both: (a) the activity sheet's "@ price" line used the whole-dollar formatter — the Build-44 cents-precision rule (prices always show cents) was applied to the detail page but this sheet was missed; (b) two words for one concept — the account page and this sheet both say Activity, the button drifted to History.</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>FIXED same hour: prices in the activity sheet are cents-precise ($250.10, never $250), and the button now says Activity — one concept, one word, pinned. Rides Build 48.</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>FIXED — verify on 48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Holding screen FULL redesign mocked (finding 6 v2, founder ask): price→graph→table grammar through the whole page, priced + unpriced states, all sections carried
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -2198,12 +2198,12 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>MOCKED to your exact order: mockups/build47-batch1/holding-detail-hero-v1-2026-07-31.html (real arithmetic, tabular numerals, everything below the hero untouched). Approve the picture and it builds into Build 48.</t>
+          <t>MOCKED v2 (FULL SCREEN per your follow-up): mockups/build47-batch1/holding-detail-full-v2-2026-07-31.html — your price→graph→table order carried through the whole page, both data states (priced + unpriced LCTX), every existing section kept in one table grammar. Approve and it builds into Build 48.</t>
         </is>
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
-          <t>MOCKED — awaiting your approval</t>
+          <t>MOCKED v2 — awaiting your approval</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B47 finding 7 BUILT (class-slice view: portion hero + class-only holdings + whole-account door; NW split rows pass class) + finding 9 answered (capped-returns label) — 1,331 green
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -2020,7 +2020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2223,12 +2223,12 @@
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>MOCKED: mockups/build47-batch1/account-class-view-v1-2026-07-31.html — slice tap lands on the class-only view (portion hero, that class's holdings summing visibly, whole account one tap away; account taps elsewhere unchanged). Approve and it builds into Build 48.</t>
-        </is>
-      </c>
-      <c r="E8" s="19" t="inlineStr">
-        <is>
-          <t>MOCKED — awaiting your approval</t>
+          <t>APPROVED + BUILT same day: tapping a class slice of a SPLIT account opens the class-only view (portion hero, that class's holdings, "See the whole account ›" one tap up; account taps elsewhere unchanged). Pinned. Rides Build 48.</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>BUILT — verify on 48</t>
         </is>
       </c>
     </row>
@@ -2254,6 +2254,31 @@
       <c r="E9" s="17" t="inlineStr">
         <is>
           <t>FIXED — verify on 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="96" customHeight="1">
+      <c r="A10" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Winners &amp; Laggards: LCTX says "since you bought" but the other stocks don't — is it because they were bought over a year ago?</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>EXACTLY RIGHT — not a bug, the capped-returns honesty rule you approved in July: a holding bought more recently than the selected window is measured from YOUR purchase date and labeled; holdings held longer show the plain window return. The market comparison always uses the same dates as your side.</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>No change — answered. The ⓘ on "How these numbers work" carries your approved explanation.</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>ANSWERED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B47 finding 11: debt model gaps verified (drifted editors, no installment end-date, due-in-full unrepresentable) — repayment-shaped editor mocked; findings tab current
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -2020,7 +2020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2279,6 +2279,56 @@
       <c r="E10" s="17" t="inlineStr">
         <is>
           <t>ANSWERED</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="128" customHeight="1">
+      <c r="A11" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Cash-flow Income tab: two add-income entries and a sentence explaining what a button will ask — "app is explaining something not relevant on that screen"</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>RIGHT — and the critique lands on my own day-old fix: I made the explanation plainer when the answer was to DELETE the explanation and merge the entries. Screens offer actions; they don't narrate them.</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>FIXED same hour: ONE "＋ Add income ›" entry, zero explanatory sentences — the chooser (Salary / Stock vesting / Rental / Self-employment) carries the meaning, and each choice deep-links straight into its editor. Rides Build 48.</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>FIXED — verify on 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="128" customHeight="1">
+      <c r="A12" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Cash-flow Debts: asks min payment + due day — no mortgage end year, no actual-monthly-payment; and a personal loan due IN FULL in 5 months cannot be entered at all</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>VERIFIED, three layers: (a) the Cash-flow Debts editor asks fewer fields than the Net-worth debt editor (two editors drifted — the min-AND-you-pay fields exist only on Net worth); (b) NO editor captures an installment end date — the credit-card framing was applied to mortgages; (c) the due-in-full structure does not exist in the model — your 5-month balloon loan is unrepresentable, and the closest fit misstates reality as a monthly minimum.</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>MOCKED: mockups/build47-batch1/debt-editor-v1-2026-07-31.html — ONE editor shaped by repayment: installment (real payment ↔ paid-off-by, either computed from the other) · revolving (today's fields) · due in full (amount + date → lands in Cash flow's big-ticket radar and the bill calendar). Model change touches payoff/DTI/plan — builds after your approval.</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>MOCKED — awaiting your approval</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
User-test results workbook (152 cases, all PASS) + honest payload statuses
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1430,7 +1430,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BUILT — 1366 green</t>
+          <t>BUILT — 1367 green</t>
         </is>
       </c>
     </row>
@@ -1445,7 +1445,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BUILT — 1366 green</t>
+          <t>BUILT — 1367 green</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TO BUILD — in 48</t>
+          <t>NOT BUILT YET — approved; next up</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TO BUILD — in 48</t>
+          <t>BUILT (9 of 10) — A1,2,4,5,6,7,8,9,10 done; A3 bonus-MONTH editor still to add</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TO BUILD — in 48</t>
+          <t>PARTIAL — verb sweep ✓, menu trim ✓, voice ×3 ✓, 4% reword ✓ · SS remind-me, goal-offtrack insight, Add-something-else link NOT BUILT YET</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DOCS — may trail the cut</t>
+          <t>NOT STARTED — docs trail the cut</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fresh gates + user-test results 2026-08-03 (158 PASS) + payload statuses final
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1430,7 +1430,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BUILT — 1367 green</t>
+          <t>BUILT</t>
         </is>
       </c>
     </row>
@@ -1445,7 +1445,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BUILT — 1367 green</t>
+          <t>BUILT</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>NOT BUILT YET — approved; next up</t>
+          <t>BUILT — capture + sim + hub rows, 6 pins</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BUILT (9 of 10) — A1,2,4,5,6,7,8,9,10 done; A3 bonus-MONTH editor still to add</t>
+          <t>BUILT — 10 of 10</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PARTIAL — verb sweep ✓, menu trim ✓, voice ×3 ✓, 4% reword ✓ · SS remind-me, goal-offtrack insight, Add-something-else link NOT BUILT YET</t>
+          <t>BUILT — all 7 decision items</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1520,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MOCK-FIRST — next batch</t>
+          <t>MOCKED — return-breakdown-v1 awaiting verdict (does NOT block 48)</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>NOT STARTED — docs trail the cut</t>
+          <t>DONE — PRD amendments tab, UX rows, design rows, flows v2</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ON HOLD — founder evaluating</t>
+          <t>ON HOLD — founder evaluating providers</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B48 walk finding 1: first-run bullet names the account kinds (investment, 401k, checking, savings, etc.)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -18,6 +18,7 @@
     <sheet name="PRD v1.1" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Build 47 — plan" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Build 48 — payload" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Build 48 — findings" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1559,6 +1560,72 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Your finding</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Verified root cause</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>Setup screen, first bullet: "every account" — name the kinds: account (investment, 401k, checking, savings, etc.)</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>The first-run bullet said "every account, debt, and dollar" without examples — a 55-70 first-timer shouldn't have to guess what counts.</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>FIXED same hour: bullet now reads "every account (investment, 401k, checking, savings, etc.), debt, and dollar in one live view." Rides Build 49.</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>FIXED — verify on 49</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
B48 walk finding 2: class-view addition line now sums ONLY the viewed class (was whole-account) — my A8 fidelity-pass bug; pinned
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1566,7 +1566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1616,6 +1616,31 @@
         </is>
       </c>
       <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>FIXED — verify on 49</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="96" customHeight="1">
+      <c r="A3" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Class-view addition line: "$224,690 + 63,405 + 60,400 + 4,235 + 1,080 + 838 + 504 = 838" — the sum is nonsense</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>MY BUG (introduced in the pre-48 audit fidelity pass, 3 days old): the visible list filters to the class you tapped, but the addition line I added beneath it summed EVERY holding in the account while the "=" showed only the tapped slice's total. Your seven numbers = the whole Vanguard account; 838 = the slice you were on.</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>FIXED same hour: the addition uses exactly the same class filter as the list — only the viewed slice's holdings appear, and the equality holds by construction. Pinned with a mixed connected-account test (the stock row can never leak into the bonds sum again). Rides Build 49.</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>FIXED — verify on 49</t>
         </is>

</xml_diff>

<commit_message>
B48 findings 3+4: holding rows on the account page open THE holding page (one thing, one page); '✎ Edit' readable; finding 5 (CD classification) logged OPEN
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1566,7 +1566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1643,6 +1643,81 @@
       <c r="E3" s="17" t="inlineStr">
         <is>
           <t>FIXED — verify on 49</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="84" customHeight="1">
+      <c r="A4" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Tapping LCTX from Invest opens its full page; tapping the same LCTX line inside the account page does nothing — same name, different behavior</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>RIGHT — the account page listed holdings as print-only rows. One investment should have ONE page, reachable from every door.</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>FIXED same hour: every holding row on the account page (whole view AND class view) now opens the same holding page Invest opens. Cash and option rows stay print-only (they have no page). Rides Build 49.</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>FIXED — verify on 49</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="84" customHeight="1">
+      <c r="A5" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>The ✎ edit mark top-right of the holding page is tiny and hard to see</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>RIGHT — a lone pencil glyph at link size. Too small for anyone, not just 55-70 eyes.</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>FIXED same hour: it now reads "✎ Edit" at the same size and weight as the Back link. Rides Build 49.</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>FIXED — verify on 49</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="84" customHeight="1">
+      <c r="A6" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Imported CD sits under Cash and cash equivalents; the Vanguard CD sits under Bonds &amp; CDs</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>CONFIRMED inconsistency: standalone CDs are sorted by maturity (under 1 year = cash, longer = bond) but the file import never asks for a maturity date, so it guessed. CDs inside a brokerage always count as bonds.</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>Today: edit the imported CD and set its maturity date — it re-sorts itself. Proper fix (your word pending): the import asks for the maturity whenever it sees a CD.</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>OPEN — your call on the import fix</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B48 findings 6-9 logged OPEN (CD maturity in name, naming rule, freshness wording, institution data shapes) — research-first per founder order
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1566,7 +1566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1718,6 +1718,106 @@
       <c r="E6" s="19" t="inlineStr">
         <is>
           <t>OPEN — your call on the import fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="78" customHeight="1">
+      <c r="A7" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Imported CD carries its maturity (8-24-26) IN ITS NAME, but Edit offers only name/value — no maturity field</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>CONFIRMED: the import never captures maturity, and the imported holding's edit path has no maturity field — even though the date is sitting in the description text.</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>AWAITING RESEARCH (your order): fix will read the date out of the description automatically + add the maturity field to edit.</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>OPEN — research first</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="78" customHeight="1">
+      <c r="A8" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Vanguard stocks list as ONE line (Vanguard - Brokerage) under Stocks/ETFs; the E*TRADE stock lists as "Etrade LCTX"</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>CONFIRMED: connected accounts keep the broker's account name; the file import names a single-stock file BY ITS TICKER. Different door, different naming rule.</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>AWAITING RESEARCH: one naming rule (institution + account type; never a ticker as an account name).</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>OPEN — research first</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="78" customHeight="1">
+      <c r="A9" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Freshness wording differs: "Imported 2026-08-03" vs "Connected · updated today"</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>CONFIRMED: two formats for the same concept.</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>AWAITING RESEARCH BATCH: one wording (relative words: today / yesterday / N days ago) everywhere.</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>OPEN — research first</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="78" customHeight="1">
+      <c r="A10" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>By class vs By type unclear; and under By type Vanguard stays ONE account while E*TRADE splits into several</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>CONFIRMED ROOT CAUSE (your diagnosis): E*TRADE the institution delivers MULTIPLE internal accounts (brokerage + sweep etc.); Vanguard delivers one. By-type groups whole accounts by their kind, so E*TRADE's pieces land under different types. The app must normalize institution data shapes, not mirror them.</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>AWAITING RESEARCH: per-institution data-shape report → normalization rules → then the fix set as one batch.</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>OPEN — research first</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Findings 5-9 batch, slice 1: savings->brokerage rule-6 correction (heals founder's E*TRADE type), CD maturity editable on the edit sheet (re-sorts class), ticker-as-name ban; 3 pins
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -1712,12 +1712,12 @@
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>Today: edit the imported CD and set its maturity date — it re-sorts itself. Proper fix (your word pending): the import asks for the maturity whenever it sees a CD.</t>
+          <t>PARTIAL BUILD: editing a CD/bond account now exposes its maturity date, and the date re-sorts the class by the one rule (under 1 yr = cash · 1 yr+ = bond). STILL TO BUILD in this batch: reading the date out of the name text automatically (import + connected), the import asking for maturity on CDs.</t>
         </is>
       </c>
       <c r="E6" s="19" t="inlineStr">
         <is>
-          <t>OPEN — your call on the import fix</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
     </row>
@@ -1762,12 +1762,12 @@
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>AWAITING RESEARCH: one naming rule (institution + account type; never a ticker as an account name).</t>
+          <t>PARTIAL BUILD: the import no longer names an account after a ticker (rule 1). STILL TO BUILD: full institution+type naming sweep.</t>
         </is>
       </c>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>OPEN — research first</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
     </row>
@@ -1812,12 +1812,12 @@
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>AWAITING RESEARCH: per-institution data-shape report → normalization rules → then the fix set as one batch.</t>
+          <t>PARTIAL BUILD: rule-6 case built — a "savings"-typed account from the brokerage-only pipe now maps to BROKERAGE (not confident → the account-type question can still fix IRAs); your mistyped E*TRADE account heals on next sync. STILL TO BUILD: institution grouping presentation.</t>
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>OPEN — research first</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
     </row>

</xml_diff>